<commit_message>
Correct XuanYuanDevPlatform path to E drive
</commit_message>
<xml_diff>
--- a/codex_tasks/艾尔登法环_第一二大陆_Codex施工包_20260821/项目档案/02_已确认规则与数值.xlsx
+++ b/codex_tasks/艾尔登法环_第一二大陆_Codex施工包_20260821/项目档案/02_已确认规则与数值.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R0b16e4957d6343f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="已确认规则" sheetId="2" r:id="R683c277bfea440d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数值参数" sheetId="3" r:id="R569e76d2edce4693"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="装备索引" sheetId="4" r:id="R58324e00c019482b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="怪物索引" sheetId="5" r:id="R5ab8d09e2f384701"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="地图索引" sheetId="6" r:id="Rb1d9da1718924c46"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="掉落索引" sheetId="7" r:id="R5c349caf78124be2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="Rf7ab3d8a9d534635"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="已确认规则" sheetId="2" r:id="R6c05587e50584d60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数值参数" sheetId="3" r:id="Rbc3c498554244fa0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="装备索引" sheetId="4" r:id="R31985d280cdc4538"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="怪物索引" sheetId="5" r:id="Rd3787ced0beb4919"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="地图索引" sheetId="6" r:id="Rb52ed0867d7849c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="掉落索引" sheetId="7" r:id="Rc30af1473fc24785"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -248,7 +248,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="67">
+  <x:cellXfs count="68">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -410,6 +410,9 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -5502,7 +5505,7 @@
         <x:v>施工交付</x:v>
       </x:c>
       <x:c r="C201" s="62" t="str">
-        <x:v>第一、第二大陆怪物与装备修改表由当前窗口制作，交给能访问D:\MirServer与D:\XuanYuanDevPlatform的服务端Codex窗口备份、测试导入和进服实测；偏差超过15%停止生产导入。</x:v>
+        <x:v>第一、第二大陆怪物与装备修改表由当前窗口制作，交给能访问D:\MirServer与E:\XuanYuanDevPlatform的服务端Codex窗口备份、测试导入和进服实测；偏差超过15%停止生产导入。</x:v>
       </x:c>
       <x:c r="D201" s="62" t="str">
         <x:v>工作流已确认</x:v>
@@ -5515,6 +5518,29 @@
       </x:c>
       <x:c r="G201" s="63" t="str">
         <x:v>追梦六件只按名称覆盖数值，不覆盖用户本机时装首饰盒部位</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="202" ht="44" customHeight="1">
+      <x:c r="A202" s="64" t="str">
+        <x:v>EL-PLATFORM-PATH-001</x:v>
+      </x:c>
+      <x:c r="B202" s="65" t="str">
+        <x:v>施工路径</x:v>
+      </x:c>
+      <x:c r="C202" s="65" t="str">
+        <x:v>开发平台正式目录为E:\XuanYuanDevPlatform；旧D:\XuanYuanDevPlatform已迁移并失效。服务端D:\MirServer及任务目录保持不变。</x:v>
+      </x:c>
+      <x:c r="D202" s="65" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="E202" s="67" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="F202" s="65" t="str">
+        <x:v>用户2026-08-22纠正</x:v>
+      </x:c>
+      <x:c r="G202" s="66" t="str">
+        <x:v>替代所有旧D盘平台执行口径；只修正路径，不改变施工数值与15%实测门槛</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Archive NPC economy roles and combat framework
</commit_message>
<xml_diff>
--- a/codex_tasks/艾尔登法环_第一二大陆_Codex施工包_20260821/项目档案/02_已确认规则与数值.xlsx
+++ b/codex_tasks/艾尔登法环_第一二大陆_Codex施工包_20260821/项目档案/02_已确认规则与数值.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="Rf7ab3d8a9d534635"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="已确认规则" sheetId="2" r:id="R6c05587e50584d60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数值参数" sheetId="3" r:id="Rbc3c498554244fa0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="装备索引" sheetId="4" r:id="R31985d280cdc4538"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="怪物索引" sheetId="5" r:id="Rd3787ced0beb4919"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="地图索引" sheetId="6" r:id="Rb52ed0867d7849c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="掉落索引" sheetId="7" r:id="Rc30af1473fc24785"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R39638f2021c048ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="已确认规则" sheetId="2" r:id="R5156065866b84c55"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数值参数" sheetId="3" r:id="R07c86cedbdd648df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="装备索引" sheetId="4" r:id="Rd06aef7167eb42e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="怪物索引" sheetId="5" r:id="R8658d2cdef5b42fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="地图索引" sheetId="6" r:id="R52a5405cf07a45c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="掉落索引" sheetId="7" r:id="R07f5c0e53cbf4c16"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -248,7 +248,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="68">
+  <x:cellXfs count="71">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -413,6 +413,15 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="6" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2374,22 +2383,22 @@
         <x:v>EL-ECO-003</x:v>
       </x:c>
       <x:c r="B65" s="30" t="str">
-        <x:v>快速毕业覆盖</x:v>
+        <x:v>经济闭环</x:v>
       </x:c>
       <x:c r="C65" s="30" t="str">
-        <x:v>满充值玩家追求同期快速毕业时，自产与装备回收合计目标只覆盖总需求约30%—50%。</x:v>
+        <x:v>按目标进度推进时，玩家自身体系的打怪、直接掉落与装备回收合计只覆盖对应NPC阶段总需求约30%—40%。</x:v>
       </x:c>
       <x:c r="D65" s="30" t="str">
         <x:v>已确认</x:v>
       </x:c>
       <x:c r="E65" s="33" t="n">
-        <x:v>46242</x:v>
+        <x:v>46256</x:v>
       </x:c>
       <x:c r="F65" s="30" t="str">
-        <x:v>2026-08-08用户确认</x:v>
+        <x:v>用户2026-08-22最新确认</x:v>
       </x:c>
       <x:c r="G65" s="30" t="str">
-        <x:v>其余依靠玩家交易收购</x:v>
+        <x:v>其余60%—70%依靠向其他玩家购买；替代旧30%—50%口径</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="15" hidden="0" customHeight="1">
@@ -4352,22 +4361,22 @@
         <x:v>EL-EQUIP-CODEX-WORKFLOW</x:v>
       </x:c>
       <x:c r="B151" s="30" t="str">
-        <x:v>装备施工</x:v>
+        <x:v>施工分工</x:v>
       </x:c>
       <x:c r="C151" s="30" t="str">
-        <x:v>装备调整由助手通过Codex制作平台可导入修改表，用户审核后导入；未经审核的机械拼接名称不得入库。</x:v>
+        <x:v>怪物与装备调整由当前窗口严格按平台最新模板制作修改表，用户自行审核并通过平台导入；不再交给另一服务端Codex窗口执行。</x:v>
       </x:c>
       <x:c r="D151" s="30" t="str">
         <x:v>已确认</x:v>
       </x:c>
       <x:c r="E151" s="30" t="n">
-        <x:v>46255</x:v>
+        <x:v>46256</x:v>
       </x:c>
       <x:c r="F151" s="30" t="str">
-        <x:v>2026-08-21用户确认</x:v>
+        <x:v>用户2026-08-22最新分工</x:v>
       </x:c>
       <x:c r="G151" s="30" t="str">
-        <x:v>本轮只归档工作流，未擅自改装备数据</x:v>
+        <x:v>现有第一、第二大陆交付表保持不变</x:v>
       </x:c>
     </x:row>
     <x:row r="152" ht="15" hidden="0" customHeight="1">
@@ -4490,22 +4499,22 @@
         <x:v>EL-DATA-OWNER-001</x:v>
       </x:c>
       <x:c r="B157" s="30" t="str">
-        <x:v>数据职责</x:v>
+        <x:v>数据统筹</x:v>
       </x:c>
       <x:c r="C157" s="30" t="str">
-        <x:v>当前窗口负责全版本数据统筹与NPC规划，覆盖金币、元宝、灵符、卢恩、材料及各成长系统产销平衡。</x:v>
+        <x:v>当前窗口负责全版本数据统筹与NPC规划，覆盖金币、元宝、灵符、卢恩、材料及各成长系统产销平衡；用户指定大陆、NPC类型和数量后逐个展开。</x:v>
       </x:c>
       <x:c r="D157" s="30" t="str">
         <x:v>已确认</x:v>
       </x:c>
       <x:c r="E157" s="30" t="n">
-        <x:v>46255</x:v>
+        <x:v>46256</x:v>
       </x:c>
       <x:c r="F157" s="30" t="str">
-        <x:v>2026-08-21用户授权</x:v>
+        <x:v>用户2026-08-22最新分工</x:v>
       </x:c>
       <x:c r="G157" s="30" t="str">
-        <x:v>先反算产出与毕业需求，再定价格、掉率和概率</x:v>
+        <x:v>每个NPC必须形成阶段消耗、属性收益、来源提示与交易缺口闭环</x:v>
       </x:c>
     </x:row>
     <x:row r="158" ht="15" hidden="0" customHeight="1">
@@ -5505,19 +5514,19 @@
         <x:v>施工交付</x:v>
       </x:c>
       <x:c r="C201" s="62" t="str">
-        <x:v>第一、第二大陆怪物与装备修改表由当前窗口制作，交给能访问D:\MirServer与E:\XuanYuanDevPlatform的服务端Codex窗口备份、测试导入和进服实测；偏差超过15%停止生产导入。</x:v>
+        <x:v>第一、第二大陆怪物与装备修改表由当前窗口制作并保持现有交付版本，用户自行通过E:\XuanYuanDevPlatform审核、导入和进服实测；偏差超过15%时停止继续导入并回传实测数据。</x:v>
       </x:c>
       <x:c r="D201" s="62" t="str">
-        <x:v>工作流已确认</x:v>
+        <x:v>修改表已交付，待用户导入实测</x:v>
       </x:c>
       <x:c r="E201" s="62" t="n">
-        <x:v>46255</x:v>
+        <x:v>46256</x:v>
       </x:c>
       <x:c r="F201" s="62" t="str">
-        <x:v>CODEX_EXECUTE.md</x:v>
+        <x:v>用户2026-08-22最新分工</x:v>
       </x:c>
       <x:c r="G201" s="63" t="str">
-        <x:v>追梦六件只按名称覆盖数值，不覆盖用户本机时装首饰盒部位</x:v>
+        <x:v>追梦六件只核对数值，不覆盖用户本机时装首饰盒部位</x:v>
       </x:c>
     </x:row>
     <x:row r="202" ht="44" customHeight="1">
@@ -5541,6 +5550,121 @@
       </x:c>
       <x:c r="G202" s="66" t="str">
         <x:v>替代所有旧D盘平台执行口径；只修正路径，不改变施工数值与15%实测门槛</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="203" ht="44" customHeight="1">
+      <x:c r="A203" s="55" t="str">
+        <x:v>EL-USER-IMPORT-001</x:v>
+      </x:c>
+      <x:c r="B203" s="56" t="str">
+        <x:v>施工分工</x:v>
+      </x:c>
+      <x:c r="C203" s="56" t="str">
+        <x:v>当前窗口负责按平台最新格式填写需要修改的怪物与装备表；用户负责审核并通过E:\XuanYuanDevPlatform导入，不再另行制作执行单转交其他Codex窗口。</x:v>
+      </x:c>
+      <x:c r="D203" s="56" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="E203" s="68" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="F203" s="56" t="str">
+        <x:v>用户2026-08-22最新分工</x:v>
+      </x:c>
+      <x:c r="G203" s="57" t="str">
+        <x:v>本次不修改已交付的五份怪物、装备及资源NPC总账</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="204" ht="44" customHeight="1">
+      <x:c r="A204" s="58" t="str">
+        <x:v>EL-NPC-SPEC-001</x:v>
+      </x:c>
+      <x:c r="B204" s="59" t="str">
+        <x:v>NPC规划</x:v>
+      </x:c>
+      <x:c r="C204" s="59" t="str">
+        <x:v>用户指定各大陆需要的成长或合成NPC类型与数量；当前窗口逐个给出NPC名称、小情节、开放阶段、当前级到目标级、消耗货币、消耗材料、提升属性或合成结果、材料来源与玩家提示。</x:v>
+      </x:c>
+      <x:c r="D204" s="59" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="E204" s="69" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="F204" s="59" t="str">
+        <x:v>用户2026-08-22最新分工</x:v>
+      </x:c>
+      <x:c r="G204" s="60" t="str">
+        <x:v>必须严格按用户给出的大陆分布展开，不擅自新增系统</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="205" ht="44" customHeight="1">
+      <x:c r="A205" s="58" t="str">
+        <x:v>EL-NPC-MARKET-001</x:v>
+      </x:c>
+      <x:c r="B205" s="59" t="str">
+        <x:v>经济闭环</x:v>
+      </x:c>
+      <x:c r="C205" s="59" t="str">
+        <x:v>每个NPC阶段总需求都要单独核算：玩家自身打怪、掉落与回收合计仅覆盖约30%—40%，其余60%—70%通过玩家交易获得。</x:v>
+      </x:c>
+      <x:c r="D205" s="59" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="E205" s="69" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="F205" s="59" t="str">
+        <x:v>用户2026-08-22最新确认</x:v>
+      </x:c>
+      <x:c r="G205" s="60" t="str">
+        <x:v>适用于称号、装备合成、转生、技能、洗练、开光、锻体等消耗口</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="206" ht="44" customHeight="1">
+      <x:c r="A206" s="58" t="str">
+        <x:v>EL-FRAMEWORK-CORE-001</x:v>
+      </x:c>
+      <x:c r="B206" s="59" t="str">
+        <x:v>数值框架</x:v>
+      </x:c>
+      <x:c r="C206" s="59" t="str">
+        <x:v>底层数值区分固定值、同类加算百分比、独立乘区、概率属性与上限；同名百分比先加算，不同乘区再相乘。怪物HP按标准角色实测DPS×目标击杀时间反算，怪物攻击按人物实际承伤并扣除固定回血、周期回血与吸血后的净生存压力反算。</x:v>
+      </x:c>
+      <x:c r="D206" s="59" t="str">
+        <x:v>规划框架（具体顺序待实测）</x:v>
+      </x:c>
+      <x:c r="E206" s="69" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="F206" s="59" t="str">
+        <x:v>三份2026-07-26／28旧MD提取的基本框架</x:v>
+      </x:c>
+      <x:c r="G206" s="60" t="str">
+        <x:v>标准角色快照应包含装备、称号、转生、锻体、洗练、赞助及外部成长；固定切割、处决、首刀/末刀等特殊伤害单列</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="207" ht="44" customHeight="1">
+      <x:c r="A207" s="61" t="str">
+        <x:v>EL-LEGACY-MD-BOUNDARY-001</x:v>
+      </x:c>
+      <x:c r="B207" s="62" t="str">
+        <x:v>旧档边界</x:v>
+      </x:c>
+      <x:c r="C207" s="62" t="str">
+        <x:v>三份2026-07-26／28旧MD只用于补充底层属性类型、乘区分类、标准角色快照和DPS/TTK/净承伤反算框架；其中具体数值、旧成长路线和旧NPC方案均不恢复。</x:v>
+      </x:c>
+      <x:c r="D207" s="62" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="E207" s="70" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="F207" s="62" t="str">
+        <x:v>用户2026-08-22最新澄清</x:v>
+      </x:c>
+      <x:c r="G207" s="63" t="str">
+        <x:v>禁止恢复旧64列表、武器幸运9、赞助基础爆率200%、每转神力0.05、23000灵符费用及旧图鉴/称号/NPC路线</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Archive dual code databases and collection drop rules
</commit_message>
<xml_diff>
--- a/codex_tasks/艾尔登法环_第一二大陆_Codex施工包_20260821/项目档案/02_已确认规则与数值.xlsx
+++ b/codex_tasks/艾尔登法环_第一二大陆_Codex施工包_20260821/项目档案/02_已确认规则与数值.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R39638f2021c048ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="已确认规则" sheetId="2" r:id="R5156065866b84c55"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数值参数" sheetId="3" r:id="R07c86cedbdd648df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="装备索引" sheetId="4" r:id="Rd06aef7167eb42e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="怪物索引" sheetId="5" r:id="R8658d2cdef5b42fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="地图索引" sheetId="6" r:id="R52a5405cf07a45c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="掉落索引" sheetId="7" r:id="R07f5c0e53cbf4c16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R6446056a14f640fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="已确认规则" sheetId="2" r:id="Rd1fbdabbe69a45c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数值参数" sheetId="3" r:id="R59f33df46d8c474e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="装备索引" sheetId="4" r:id="R44c29155dc8343f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="怪物索引" sheetId="5" r:id="R6009d03528ef4086"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="地图索引" sheetId="6" r:id="R32e05209d3a04f56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="掉落索引" sheetId="7" r:id="Rb3524c81cf754343"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5667,6 +5667,167 @@
         <x:v>禁止恢复旧64列表、武器幸运9、赞助基础爆率200%、每转神力0.05、23000灵符费用及旧图鉴/称号/NPC路线</x:v>
       </x:c>
     </x:row>
+    <x:row r="208" ht="44" customHeight="1">
+      <x:c r="A208" s="55" t="str">
+        <x:v>EL-CODEDB-EQUIP-001</x:v>
+      </x:c>
+      <x:c r="B208" s="56" t="str">
+        <x:v>编码底账</x:v>
+      </x:c>
+      <x:c r="C208" s="56" t="str">
+        <x:v>装备编码库现行原件为/传奇私服之旅/装备素材套装代码表.xlsx，以“全资源索引”为唯一检索入口；已核验1075条唯一代码、重复0、Items/StateItem/DnItems三库同码异常0。</x:v>
+      </x:c>
+      <x:c r="D208" s="56" t="str">
+        <x:v>已确认并核验</x:v>
+      </x:c>
+      <x:c r="E208" s="68" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="F208" s="56" t="str">
+        <x:v>装备编码库原件＋2026-08-22复核</x:v>
+      </x:c>
+      <x:c r="G208" s="57" t="str">
+        <x:v>不得凭聊天摘要或代码范围重建；新增来源编号前先查原件与现行占用</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="209" ht="44" customHeight="1">
+      <x:c r="A209" s="58" t="str">
+        <x:v>EL-CODEDB-MATERIAL-001</x:v>
+      </x:c>
+      <x:c r="B209" s="59" t="str">
+        <x:v>编码底账</x:v>
+      </x:c>
+      <x:c r="C209" s="59" t="str">
+        <x:v>材料编码库与装备编码库分开长期维护；材料物品ID、数据库Idx、Items背包图标Looks及用途映射以材料库原件为准，两库不得合并、互推或只保存摘要。</x:v>
+      </x:c>
+      <x:c r="D209" s="59" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="E209" s="69" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="F209" s="59" t="str">
+        <x:v>用户2026-08-22要求完整继承</x:v>
+      </x:c>
+      <x:c r="G209" s="60" t="str">
+        <x:v>材料只使用Items图库时仍须独立登记，不从装备来源编号反推</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="210" ht="44" customHeight="1">
+      <x:c r="A210" s="58" t="str">
+        <x:v>EL-MAT-IMPORT-65-001</x:v>
+      </x:c>
+      <x:c r="B210" s="59" t="str">
+        <x:v>材料事务</x:v>
+      </x:c>
+      <x:c r="C210" s="59" t="str">
+        <x:v>65件材料事务：图标65/65，Items Looks 6398—6462；数据库65/65，Idx 907—971；972—983预留0行；793/794/802保持不变。材料未写DnItems或StateItem。</x:v>
+      </x:c>
+      <x:c r="D210" s="59" t="str">
+        <x:v>事务已确认，原件待接续</x:v>
+      </x:c>
+      <x:c r="E210" s="69" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="F210" s="59" t="str">
+        <x:v>截图事务凭证</x:v>
+      </x:c>
+      <x:c r="G210" s="60" t="str">
+        <x:v>Git d9f705fbe8da4a017038568f9f8d5cbd1b504748；XYMI-20260822-013718-C9646062；XYMD-20260822-014350-1C7690A1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="211" ht="44" customHeight="1">
+      <x:c r="A211" s="58" t="str">
+        <x:v>EL-MAT-ALLOC-FREEZE-001</x:v>
+      </x:c>
+      <x:c r="B211" s="59" t="str">
+        <x:v>材料施工</x:v>
+      </x:c>
+      <x:c r="C211" s="59" t="str">
+        <x:v>在65条逐行材料数据库原件接续前，Idx 907—971及Items Looks 6398—6462按已占用冻结，Idx 972—983按预留冻结；不新增材料编号，不把事务摘要冒充完整材料库。</x:v>
+      </x:c>
+      <x:c r="D211" s="59" t="str">
+        <x:v>立即生效</x:v>
+      </x:c>
+      <x:c r="E211" s="69" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="F211" s="59" t="str">
+        <x:v>用户2026-08-22要求完整继承</x:v>
+      </x:c>
+      <x:c r="G211" s="60" t="str">
+        <x:v>同数字Looks段与装备资源库暂列原件级核验项，不在缺少WZL差异时擅自判冲突或改号</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="212" ht="44" customHeight="1">
+      <x:c r="A212" s="58" t="str">
+        <x:v>EL-DREAM-POOL-001</x:v>
+      </x:c>
+      <x:c r="B212" s="59" t="str">
+        <x:v>掉落机制</x:v>
+      </x:c>
+      <x:c r="C212" s="59" t="str">
+        <x:v>六件追梦神器是极低爆率终极特殊装备，第二大陆及以后所有怪物共用一次1/x RANDOM公共奖池判定，基础x按几十万至百万量级规划；触发后再从6件中随机出现1件。人物爆率倍率作用于基础判定；1/10000配100倍人物爆率时约100杀触发一次奖池。</x:v>
+      </x:c>
+      <x:c r="D212" s="59" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="E212" s="69" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="F212" s="59" t="str">
+        <x:v>用户2026-08-22最新澄清</x:v>
+      </x:c>
+      <x:c r="G212" s="60" t="str">
+        <x:v>禁止六件分别独立判定；单件期望再按池内权重计算</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="213" ht="44" customHeight="1">
+      <x:c r="A213" s="58" t="str">
+        <x:v>EL-COLLECT-CMD-001</x:v>
+      </x:c>
+      <x:c r="B213" s="59" t="str">
+        <x:v>收集图鉴</x:v>
+      </x:c>
+      <x:c r="C213" s="59" t="str">
+        <x:v>专属装备收集图鉴由命令触发脚本处理，不设置独立NPC；当前窗口提供单件收集奖励及大陆全部装备收集奖励表。</x:v>
+      </x:c>
+      <x:c r="D213" s="59" t="str">
+        <x:v>结构已确认，数值待定</x:v>
+      </x:c>
+      <x:c r="E213" s="69" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="F213" s="59" t="str">
+        <x:v>用户2026-08-22最新澄清</x:v>
+      </x:c>
+      <x:c r="G213" s="60" t="str">
+        <x:v>逐件奖励、页面划分和整页处决未确认时不得猜填</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="214" ht="44" customHeight="1">
+      <x:c r="A214" s="61" t="str">
+        <x:v>EL-CONTINENT-COLLECT-001</x:v>
+      </x:c>
+      <x:c r="B214" s="62" t="str">
+        <x:v>收集图鉴</x:v>
+      </x:c>
+      <x:c r="C214" s="62" t="str">
+        <x:v>每个正式大陆另设1件不可装备、可收集的大陆专属图鉴材料，由本大陆所有怪物掉落；收集价值和奖励强度高于普通单件专属。</x:v>
+      </x:c>
+      <x:c r="D214" s="62" t="str">
+        <x:v>结构已确认，细项待定</x:v>
+      </x:c>
+      <x:c r="E214" s="70" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="F214" s="62" t="str">
+        <x:v>用户2026-08-22新增</x:v>
+      </x:c>
+      <x:c r="G214" s="63" t="str">
+        <x:v>逐大陆名称、代码、基础爆率、奖励及登记是否消耗实物待确认</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
@@ -10337,6 +10498,450 @@
         <x:v>超过15%停止生产导入并回算</x:v>
       </x:c>
     </x:row>
+    <x:row r="149" ht="44" customHeight="1">
+      <x:c r="A149" s="55" t="str">
+        <x:v>EL-PARAM-EQUIP-CODE-COUNT</x:v>
+      </x:c>
+      <x:c r="B149" s="56" t="str">
+        <x:v>编码库</x:v>
+      </x:c>
+      <x:c r="C149" s="56" t="str">
+        <x:v>装备资源索引总数</x:v>
+      </x:c>
+      <x:c r="D149" s="56" t="str">
+        <x:v>条</x:v>
+      </x:c>
+      <x:c r="E149" s="56" t="n">
+        <x:v>1075</x:v>
+      </x:c>
+      <x:c r="F149" s="56" t="n">
+        <x:v>1075</x:v>
+      </x:c>
+      <x:c r="G149" s="56" t="n">
+        <x:v>1075</x:v>
+      </x:c>
+      <x:c r="H149" s="56" t="str">
+        <x:v>已核验</x:v>
+      </x:c>
+      <x:c r="I149" s="68" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="J149" s="57" t="str">
+        <x:v>装备素材套装代码表.xlsx／全资源索引</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="150" ht="44" customHeight="1">
+      <x:c r="A150" s="58" t="str">
+        <x:v>EL-PARAM-EQUIP-CODE-DUP</x:v>
+      </x:c>
+      <x:c r="B150" s="59" t="str">
+        <x:v>编码库</x:v>
+      </x:c>
+      <x:c r="C150" s="59" t="str">
+        <x:v>装备资源代码重复数</x:v>
+      </x:c>
+      <x:c r="D150" s="59" t="str">
+        <x:v>条</x:v>
+      </x:c>
+      <x:c r="E150" s="59" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F150" s="59" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G150" s="59" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H150" s="59" t="str">
+        <x:v>已核验</x:v>
+      </x:c>
+      <x:c r="I150" s="69" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="J150" s="60" t="str">
+        <x:v>1075条唯一</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="151" ht="44" customHeight="1">
+      <x:c r="A151" s="58" t="str">
+        <x:v>EL-PARAM-EQUIP-CODE-TRILIB</x:v>
+      </x:c>
+      <x:c r="B151" s="59" t="str">
+        <x:v>编码库</x:v>
+      </x:c>
+      <x:c r="C151" s="59" t="str">
+        <x:v>Items/StateItem/DnItems三库同码异常</x:v>
+      </x:c>
+      <x:c r="D151" s="59" t="str">
+        <x:v>条</x:v>
+      </x:c>
+      <x:c r="E151" s="59" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F151" s="59" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G151" s="59" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H151" s="59" t="str">
+        <x:v>已核验</x:v>
+      </x:c>
+      <x:c r="I151" s="69" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="J151" s="60" t="str">
+        <x:v>装备库原件复核</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="152" ht="44" customHeight="1">
+      <x:c r="A152" s="58" t="str">
+        <x:v>EL-PARAM-MAT-IMPORT-COUNT</x:v>
+      </x:c>
+      <x:c r="B152" s="59" t="str">
+        <x:v>材料库</x:v>
+      </x:c>
+      <x:c r="C152" s="59" t="str">
+        <x:v>本次新增材料行数</x:v>
+      </x:c>
+      <x:c r="D152" s="59" t="str">
+        <x:v>条</x:v>
+      </x:c>
+      <x:c r="E152" s="59" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="F152" s="59" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="G152" s="59" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="H152" s="59" t="str">
+        <x:v>事务已确认，原件待接续</x:v>
+      </x:c>
+      <x:c r="I152" s="69" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="J152" s="60" t="str">
+        <x:v>数据库事务XYMD-20260822-014350-1C7690A1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="153" ht="44" customHeight="1">
+      <x:c r="A153" s="58" t="str">
+        <x:v>EL-PARAM-MAT-IDX-MIN</x:v>
+      </x:c>
+      <x:c r="B153" s="59" t="str">
+        <x:v>材料库</x:v>
+      </x:c>
+      <x:c r="C153" s="59" t="str">
+        <x:v>新增材料Idx起点</x:v>
+      </x:c>
+      <x:c r="D153" s="59" t="str">
+        <x:v>Idx</x:v>
+      </x:c>
+      <x:c r="E153" s="59" t="n">
+        <x:v>907</x:v>
+      </x:c>
+      <x:c r="F153" s="59" t="n">
+        <x:v>907</x:v>
+      </x:c>
+      <x:c r="G153" s="59" t="n">
+        <x:v>907</x:v>
+      </x:c>
+      <x:c r="H153" s="59" t="str">
+        <x:v>已占用冻结</x:v>
+      </x:c>
+      <x:c r="I153" s="69" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="J153" s="60" t="str">
+        <x:v>65条连续范围</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="154" ht="44" customHeight="1">
+      <x:c r="A154" s="58" t="str">
+        <x:v>EL-PARAM-MAT-IDX-MAX</x:v>
+      </x:c>
+      <x:c r="B154" s="59" t="str">
+        <x:v>材料库</x:v>
+      </x:c>
+      <x:c r="C154" s="59" t="str">
+        <x:v>新增材料Idx终点</x:v>
+      </x:c>
+      <x:c r="D154" s="59" t="str">
+        <x:v>Idx</x:v>
+      </x:c>
+      <x:c r="E154" s="59" t="n">
+        <x:v>971</x:v>
+      </x:c>
+      <x:c r="F154" s="59" t="n">
+        <x:v>971</x:v>
+      </x:c>
+      <x:c r="G154" s="59" t="n">
+        <x:v>971</x:v>
+      </x:c>
+      <x:c r="H154" s="59" t="str">
+        <x:v>已占用冻结</x:v>
+      </x:c>
+      <x:c r="I154" s="69" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="J154" s="60" t="str">
+        <x:v>65条连续范围</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="155" ht="44" customHeight="1">
+      <x:c r="A155" s="58" t="str">
+        <x:v>EL-PARAM-MAT-LOOKS-MIN</x:v>
+      </x:c>
+      <x:c r="B155" s="59" t="str">
+        <x:v>材料库</x:v>
+      </x:c>
+      <x:c r="C155" s="59" t="str">
+        <x:v>新增Items Looks起点</x:v>
+      </x:c>
+      <x:c r="D155" s="59" t="str">
+        <x:v>Looks</x:v>
+      </x:c>
+      <x:c r="E155" s="59" t="n">
+        <x:v>6398</x:v>
+      </x:c>
+      <x:c r="F155" s="59" t="n">
+        <x:v>6398</x:v>
+      </x:c>
+      <x:c r="G155" s="59" t="n">
+        <x:v>6398</x:v>
+      </x:c>
+      <x:c r="H155" s="59" t="str">
+        <x:v>已占用冻结</x:v>
+      </x:c>
+      <x:c r="I155" s="69" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="J155" s="60" t="str">
+        <x:v>图标事务XYMI-20260822-013718-C9646062</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="156" ht="44" customHeight="1">
+      <x:c r="A156" s="58" t="str">
+        <x:v>EL-PARAM-MAT-LOOKS-MAX</x:v>
+      </x:c>
+      <x:c r="B156" s="59" t="str">
+        <x:v>材料库</x:v>
+      </x:c>
+      <x:c r="C156" s="59" t="str">
+        <x:v>新增Items Looks终点</x:v>
+      </x:c>
+      <x:c r="D156" s="59" t="str">
+        <x:v>Looks</x:v>
+      </x:c>
+      <x:c r="E156" s="59" t="n">
+        <x:v>6462</x:v>
+      </x:c>
+      <x:c r="F156" s="59" t="n">
+        <x:v>6462</x:v>
+      </x:c>
+      <x:c r="G156" s="59" t="n">
+        <x:v>6462</x:v>
+      </x:c>
+      <x:c r="H156" s="59" t="str">
+        <x:v>已占用冻结</x:v>
+      </x:c>
+      <x:c r="I156" s="69" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="J156" s="60" t="str">
+        <x:v>65个连续背包图标</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="157" ht="44" customHeight="1">
+      <x:c r="A157" s="58" t="str">
+        <x:v>EL-PARAM-MAT-RESERVE-MIN</x:v>
+      </x:c>
+      <x:c r="B157" s="59" t="str">
+        <x:v>材料库</x:v>
+      </x:c>
+      <x:c r="C157" s="59" t="str">
+        <x:v>材料Idx预留起点</x:v>
+      </x:c>
+      <x:c r="D157" s="59" t="str">
+        <x:v>Idx</x:v>
+      </x:c>
+      <x:c r="E157" s="59" t="n">
+        <x:v>972</x:v>
+      </x:c>
+      <x:c r="F157" s="59" t="n">
+        <x:v>972</x:v>
+      </x:c>
+      <x:c r="G157" s="59" t="n">
+        <x:v>972</x:v>
+      </x:c>
+      <x:c r="H157" s="59" t="str">
+        <x:v>预留冻结／当前0行</x:v>
+      </x:c>
+      <x:c r="I157" s="69" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="J157" s="60" t="str">
+        <x:v>不得视为空闲自动分配</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="158" ht="44" customHeight="1">
+      <x:c r="A158" s="58" t="str">
+        <x:v>EL-PARAM-MAT-RESERVE-MAX</x:v>
+      </x:c>
+      <x:c r="B158" s="59" t="str">
+        <x:v>材料库</x:v>
+      </x:c>
+      <x:c r="C158" s="59" t="str">
+        <x:v>材料Idx预留终点</x:v>
+      </x:c>
+      <x:c r="D158" s="59" t="str">
+        <x:v>Idx</x:v>
+      </x:c>
+      <x:c r="E158" s="59" t="n">
+        <x:v>983</x:v>
+      </x:c>
+      <x:c r="F158" s="59" t="n">
+        <x:v>983</x:v>
+      </x:c>
+      <x:c r="G158" s="59" t="n">
+        <x:v>983</x:v>
+      </x:c>
+      <x:c r="H158" s="59" t="str">
+        <x:v>预留冻结／当前0行</x:v>
+      </x:c>
+      <x:c r="I158" s="69" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="J158" s="60" t="str">
+        <x:v>不得视为空闲自动分配</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="159" ht="44" customHeight="1">
+      <x:c r="A159" s="58" t="str">
+        <x:v>EL-PARAM-MAT-PRESERVED</x:v>
+      </x:c>
+      <x:c r="B159" s="59" t="str">
+        <x:v>材料库</x:v>
+      </x:c>
+      <x:c r="C159" s="59" t="str">
+        <x:v>保持不变的原材料Idx</x:v>
+      </x:c>
+      <x:c r="D159" s="59" t="str">
+        <x:v>Idx列表</x:v>
+      </x:c>
+      <x:c r="E159" s="59"/>
+      <x:c r="F159" s="59"/>
+      <x:c r="G159" s="59" t="str">
+        <x:v>793、794、802</x:v>
+      </x:c>
+      <x:c r="H159" s="59" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="I159" s="69" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="J159" s="60" t="str">
+        <x:v>截图事务凭证</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="160" ht="44" customHeight="1">
+      <x:c r="A160" s="58" t="str">
+        <x:v>EL-PARAM-MAT-TEST-NEW</x:v>
+      </x:c>
+      <x:c r="B160" s="59" t="str">
+        <x:v>质检</x:v>
+      </x:c>
+      <x:c r="C160" s="59" t="str">
+        <x:v>65件材料专项测试</x:v>
+      </x:c>
+      <x:c r="D160" s="59" t="str">
+        <x:v>项</x:v>
+      </x:c>
+      <x:c r="E160" s="59" t="n">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="F160" s="59" t="n">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="G160" s="59" t="n">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="H160" s="59" t="str">
+        <x:v>事务记录通过</x:v>
+      </x:c>
+      <x:c r="I160" s="69" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="J160" s="60" t="str">
+        <x:v>仍待进服实测</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="161" ht="44" customHeight="1">
+      <x:c r="A161" s="58" t="str">
+        <x:v>EL-PARAM-MAT-TEST-LEGACY</x:v>
+      </x:c>
+      <x:c r="B161" s="59" t="str">
+        <x:v>质检</x:v>
+      </x:c>
+      <x:c r="C161" s="59" t="str">
+        <x:v>原材料回归测试</x:v>
+      </x:c>
+      <x:c r="D161" s="59" t="str">
+        <x:v>项</x:v>
+      </x:c>
+      <x:c r="E161" s="59" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="F161" s="59" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="G161" s="59" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H161" s="59" t="str">
+        <x:v>事务记录通过</x:v>
+      </x:c>
+      <x:c r="I161" s="69" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="J161" s="60" t="str">
+        <x:v>793/794/802保持不变</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="162" ht="44" customHeight="1">
+      <x:c r="A162" s="61" t="str">
+        <x:v>EL-PARAM-DREAM-POOL-SIZE</x:v>
+      </x:c>
+      <x:c r="B162" s="62" t="str">
+        <x:v>掉落</x:v>
+      </x:c>
+      <x:c r="C162" s="62" t="str">
+        <x:v>追梦神器公共奖池件数</x:v>
+      </x:c>
+      <x:c r="D162" s="62" t="str">
+        <x:v>件</x:v>
+      </x:c>
+      <x:c r="E162" s="62" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F162" s="62" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="G162" s="62" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H162" s="62" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="I162" s="70" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="J162" s="63" t="str">
+        <x:v>一次触发后六选一</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:J1"/>
@@ -10949,6 +11554,32 @@
         <x:v>修改表已生成，待Codex测试执行</x:v>
       </x:c>
     </x:row>
+    <x:row r="24" ht="44" customHeight="1">
+      <x:c r="A24" s="64" t="str">
+        <x:v>EL-EQUIP-CODEDB-001</x:v>
+      </x:c>
+      <x:c r="B24" s="65" t="str">
+        <x:v>装备编码库</x:v>
+      </x:c>
+      <x:c r="C24" s="65" t="str">
+        <x:v>1075条装备外观资源索引</x:v>
+      </x:c>
+      <x:c r="D24" s="65" t="str">
+        <x:v>全项目</x:v>
+      </x:c>
+      <x:c r="E24" s="65" t="str">
+        <x:v>/传奇私服之旅/装备素材套装代码表.xlsx</x:v>
+      </x:c>
+      <x:c r="F24" s="67" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="G24" s="65" t="str">
+        <x:v>以全资源索引检索；唯一1075，重复0，三库同码异常0</x:v>
+      </x:c>
+      <x:c r="H24" s="66" t="str">
+        <x:v>原件已核验</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
@@ -12067,6 +12698,58 @@
         <x:v>审核总账已生成，正式材料表待平台模板</x:v>
       </x:c>
     </x:row>
+    <x:row r="13" ht="44" customHeight="1">
+      <x:c r="A13" s="55" t="str">
+        <x:v>EL-DROP-DREAM-POOL-001</x:v>
+      </x:c>
+      <x:c r="B13" s="56" t="str">
+        <x:v>第二大陆及以后全部怪物</x:v>
+      </x:c>
+      <x:c r="C13" s="56" t="str">
+        <x:v>六件追梦神器公共奖池</x:v>
+      </x:c>
+      <x:c r="D13" s="56" t="str">
+        <x:v>TXT 1/x RANDOM先触发一次，再从6件随机1件</x:v>
+      </x:c>
+      <x:c r="E13" s="56" t="str">
+        <x:v>待写入逐怪正式爆率TXT</x:v>
+      </x:c>
+      <x:c r="F13" s="68" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="G13" s="56" t="str">
+        <x:v>极低爆率终极特殊装备；基础x按几十万至百万量级规划；人物爆率倍率作用于1/x；禁止六件独立判定</x:v>
+      </x:c>
+      <x:c r="H13" s="57" t="str">
+        <x:v>机制已确认，逐怪x值待规划</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="44" customHeight="1">
+      <x:c r="A14" s="61" t="str">
+        <x:v>EL-MATERIAL-DB-65-001</x:v>
+      </x:c>
+      <x:c r="B14" s="62" t="str">
+        <x:v>材料数据库</x:v>
+      </x:c>
+      <x:c r="C14" s="62" t="str">
+        <x:v>新增65件材料／Items背包图标</x:v>
+      </x:c>
+      <x:c r="D14" s="62" t="str">
+        <x:v>Idx 907—971；Looks 6398—6462</x:v>
+      </x:c>
+      <x:c r="E14" s="62" t="str">
+        <x:v>实际材料库原件待从上个窗口完整成果目录接续</x:v>
+      </x:c>
+      <x:c r="F14" s="70" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="G14" s="62" t="str">
+        <x:v>972—983预留；793/794/802不变；只写Items图库</x:v>
+      </x:c>
+      <x:c r="H14" s="63" t="str">
+        <x:v>事务已确认，逐行原件缺失</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>

</xml_diff>

<commit_message>
Correct material transaction evidence
</commit_message>
<xml_diff>
--- a/codex_tasks/艾尔登法环_第一二大陆_Codex施工包_20260821/项目档案/02_已确认规则与数值.xlsx
+++ b/codex_tasks/艾尔登法环_第一二大陆_Codex施工包_20260821/项目档案/02_已确认规则与数值.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R6446056a14f640fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="已确认规则" sheetId="2" r:id="Rd1fbdabbe69a45c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数值参数" sheetId="3" r:id="R59f33df46d8c474e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="装备索引" sheetId="4" r:id="R44c29155dc8343f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="怪物索引" sheetId="5" r:id="R6009d03528ef4086"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="地图索引" sheetId="6" r:id="R32e05209d3a04f56"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="掉落索引" sheetId="7" r:id="Rb3524c81cf754343"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="Rb9ea2fdae01741dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="已确认规则" sheetId="2" r:id="R32798b0da3a84dbc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数值参数" sheetId="3" r:id="R5aeb581a34694f47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="装备索引" sheetId="4" r:id="R5a124bac72994097"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="怪物索引" sheetId="5" r:id="Rc4b803820fd748e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="地图索引" sheetId="6" r:id="R8c8aa133c91b4226"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="掉落索引" sheetId="7" r:id="R1045cd007bbd41f0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -26,7 +26,7 @@
     <x:numFmt numFmtId="203" formatCode="0.0%"/>
     <x:numFmt numFmtId="204" formatCode="0"/>
   </x:numFmts>
-  <x:fonts count="7">
+  <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -60,6 +60,11 @@
     </x:font>
     <x:font>
       <x:sz val="10"/>
+      <x:color rgb="FF1F2937"/>
+      <x:name val="Microsoft YaHei"/>
+    </x:font>
+    <x:font>
+      <x:sz val="8"/>
       <x:color rgb="FF1F2937"/>
       <x:name val="Microsoft YaHei"/>
     </x:font>
@@ -248,7 +253,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="71">
+  <x:cellXfs count="73">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -422,6 +427,12 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="6" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -5721,7 +5732,7 @@
         <x:v>材料事务</x:v>
       </x:c>
       <x:c r="C210" s="59" t="str">
-        <x:v>65件材料事务：图标65/65，Items Looks 6398—6462；数据库65/65，Idx 907—971；972—983预留0行；793/794/802保持不变。材料未写DnItems或StateItem。</x:v>
+        <x:v>65件材料事务：图标65/65，Items图库数量由6398变为6463，Looks 6398—6462；数据库65/65，Idx 907—971；972—983预留0行；793/794/802保持不变。材料未写DnItems或StateItem。</x:v>
       </x:c>
       <x:c r="D210" s="59" t="str">
         <x:v>事务已确认，原件待接续</x:v>
@@ -5730,10 +5741,10 @@
         <x:v>46256</x:v>
       </x:c>
       <x:c r="F210" s="59" t="str">
-        <x:v>截图事务凭证</x:v>
+        <x:v>20260822_0235_65材料图标与正式入库.txt</x:v>
       </x:c>
       <x:c r="G210" s="60" t="str">
-        <x:v>Git d9f705fbe8da4a017038568f9f8d5cbd1b504748；XYMI-20260822-013718-C9646062；XYMD-20260822-014350-1C7690A1</x:v>
+        <x:v>Git d9f705fbe8da4a017038568f9f8d5cbd1b504748；XYMI-20260822-013718-C9646062；XYMD-20260822-014350-1C7690A1；新专项4项＋既有材料批量13项通过</x:v>
       </x:c>
     </x:row>
     <x:row r="211" ht="44" customHeight="1">
@@ -5854,10 +5865,10 @@
     <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="52" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="16" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="46" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="38" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
@@ -10843,7 +10854,7 @@
         <x:v>46256</x:v>
       </x:c>
       <x:c r="J159" s="60" t="str">
-        <x:v>截图事务凭证</x:v>
+        <x:v>20260822_0235交班记录；实际数据库独立回读</x:v>
       </x:c>
     </x:row>
     <x:row r="160" ht="44" customHeight="1">
@@ -10854,19 +10865,19 @@
         <x:v>质检</x:v>
       </x:c>
       <x:c r="C160" s="59" t="str">
-        <x:v>65件材料专项测试</x:v>
+        <x:v>平台新专项测试</x:v>
       </x:c>
       <x:c r="D160" s="59" t="str">
         <x:v>项</x:v>
       </x:c>
       <x:c r="E160" s="59" t="n">
-        <x:v>41</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F160" s="59" t="n">
-        <x:v>41</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G160" s="59" t="n">
-        <x:v>41</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H160" s="59" t="str">
         <x:v>事务记录通过</x:v>
@@ -10875,7 +10886,7 @@
         <x:v>46256</x:v>
       </x:c>
       <x:c r="J160" s="60" t="str">
-        <x:v>仍待进服实测</x:v>
+        <x:v>交班TXT原文；此前41为截图误读</x:v>
       </x:c>
     </x:row>
     <x:row r="161" ht="44" customHeight="1">
@@ -10886,7 +10897,7 @@
         <x:v>质检</x:v>
       </x:c>
       <x:c r="C161" s="59" t="str">
-        <x:v>原材料回归测试</x:v>
+        <x:v>既有材料批量测试</x:v>
       </x:c>
       <x:c r="D161" s="59" t="str">
         <x:v>项</x:v>
@@ -10907,7 +10918,7 @@
         <x:v>46256</x:v>
       </x:c>
       <x:c r="J161" s="60" t="str">
-        <x:v>793/794/802保持不变</x:v>
+        <x:v>13项通过；793/794/802全字段不变</x:v>
       </x:c>
     </x:row>
     <x:row r="162" ht="44" customHeight="1">
@@ -10940,6 +10951,238 @@
       </x:c>
       <x:c r="J162" s="63" t="str">
         <x:v>一次触发后六选一</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="163" ht="44" customHeight="1">
+      <x:c r="A163" s="55" t="str">
+        <x:v>EL-PARAM-MAT-ITEMS-COUNT-BEFORE</x:v>
+      </x:c>
+      <x:c r="B163" s="56" t="str">
+        <x:v>材料图库</x:v>
+      </x:c>
+      <x:c r="C163" s="56" t="str">
+        <x:v>Items图库写前数量</x:v>
+      </x:c>
+      <x:c r="D163" s="56" t="str">
+        <x:v>张</x:v>
+      </x:c>
+      <x:c r="E163" s="56" t="n">
+        <x:v>6398</x:v>
+      </x:c>
+      <x:c r="F163" s="56" t="n">
+        <x:v>6398</x:v>
+      </x:c>
+      <x:c r="G163" s="56" t="n">
+        <x:v>6398</x:v>
+      </x:c>
+      <x:c r="H163" s="56" t="str">
+        <x:v>事务证据</x:v>
+      </x:c>
+      <x:c r="I163" s="68" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="J163" s="57" t="str">
+        <x:v>写前最大有效Looks为6397</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="164" ht="44" customHeight="1">
+      <x:c r="A164" s="58" t="str">
+        <x:v>EL-PARAM-MAT-ITEMS-COUNT-AFTER</x:v>
+      </x:c>
+      <x:c r="B164" s="59" t="str">
+        <x:v>材料图库</x:v>
+      </x:c>
+      <x:c r="C164" s="59" t="str">
+        <x:v>Items图库写后数量</x:v>
+      </x:c>
+      <x:c r="D164" s="59" t="str">
+        <x:v>张</x:v>
+      </x:c>
+      <x:c r="E164" s="59" t="n">
+        <x:v>6463</x:v>
+      </x:c>
+      <x:c r="F164" s="59" t="n">
+        <x:v>6463</x:v>
+      </x:c>
+      <x:c r="G164" s="59" t="n">
+        <x:v>6463</x:v>
+      </x:c>
+      <x:c r="H164" s="59" t="str">
+        <x:v>事务证据</x:v>
+      </x:c>
+      <x:c r="I164" s="69" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="J164" s="60" t="str">
+        <x:v>新增Looks 6398—6462，共65张</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="165" ht="72" customHeight="1">
+      <x:c r="A165" s="58" t="str">
+        <x:v>EL-PARAM-MAT-DB-HASH-BEFORE</x:v>
+      </x:c>
+      <x:c r="B165" s="59" t="str">
+        <x:v>材料数据库</x:v>
+      </x:c>
+      <x:c r="C165" s="59" t="str">
+        <x:v>ApexM2.DB写前SHA256</x:v>
+      </x:c>
+      <x:c r="D165" s="59" t="str">
+        <x:v>SHA256</x:v>
+      </x:c>
+      <x:c r="E165" s="59"/>
+      <x:c r="F165" s="59"/>
+      <x:c r="G165" s="71" t="str">
+        <x:v>619C32B497530F46251FD962A71E7D8329905EE37EA5EBBCB4BF4E1E3AE41F61</x:v>
+      </x:c>
+      <x:c r="H165" s="59" t="str">
+        <x:v>事务证据</x:v>
+      </x:c>
+      <x:c r="I165" s="69" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="J165" s="60" t="str">
+        <x:v>数据库事务XYMD-20260822-014350-1C7690A1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="166" ht="72" customHeight="1">
+      <x:c r="A166" s="58" t="str">
+        <x:v>EL-PARAM-MAT-DB-HASH-AFTER</x:v>
+      </x:c>
+      <x:c r="B166" s="59" t="str">
+        <x:v>材料数据库</x:v>
+      </x:c>
+      <x:c r="C166" s="59" t="str">
+        <x:v>ApexM2.DB写后SHA256</x:v>
+      </x:c>
+      <x:c r="D166" s="59" t="str">
+        <x:v>SHA256</x:v>
+      </x:c>
+      <x:c r="E166" s="59"/>
+      <x:c r="F166" s="59"/>
+      <x:c r="G166" s="71" t="str">
+        <x:v>F683DF3AE187489ACDB482F9E6D703C5600F45F67A7F9FAC0C762EBCAA7B348B</x:v>
+      </x:c>
+      <x:c r="H166" s="59" t="str">
+        <x:v>事务证据</x:v>
+      </x:c>
+      <x:c r="I166" s="69" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="J166" s="60" t="str">
+        <x:v>65条数据库独立回读通过</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="167" ht="72" customHeight="1">
+      <x:c r="A167" s="58" t="str">
+        <x:v>EL-PARAM-MAT-WZL-HASH-BEFORE</x:v>
+      </x:c>
+      <x:c r="B167" s="59" t="str">
+        <x:v>材料图库</x:v>
+      </x:c>
+      <x:c r="C167" s="59" t="str">
+        <x:v>Items.wzl写前SHA256</x:v>
+      </x:c>
+      <x:c r="D167" s="59" t="str">
+        <x:v>SHA256</x:v>
+      </x:c>
+      <x:c r="E167" s="59"/>
+      <x:c r="F167" s="59"/>
+      <x:c r="G167" s="71" t="str">
+        <x:v>E855C1E8ECE7E8A1A4EA0C559B918A841AA12E8FDF3F06704357F46CA69FFD9C</x:v>
+      </x:c>
+      <x:c r="H167" s="59" t="str">
+        <x:v>事务证据</x:v>
+      </x:c>
+      <x:c r="I167" s="69" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="J167" s="60" t="str">
+        <x:v>图标事务XYMI-20260822-013718-C9646062</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="168" ht="72" customHeight="1">
+      <x:c r="A168" s="58" t="str">
+        <x:v>EL-PARAM-MAT-WZL-HASH-AFTER</x:v>
+      </x:c>
+      <x:c r="B168" s="59" t="str">
+        <x:v>材料图库</x:v>
+      </x:c>
+      <x:c r="C168" s="59" t="str">
+        <x:v>Items.wzl写后SHA256</x:v>
+      </x:c>
+      <x:c r="D168" s="59" t="str">
+        <x:v>SHA256</x:v>
+      </x:c>
+      <x:c r="E168" s="59"/>
+      <x:c r="F168" s="59"/>
+      <x:c r="G168" s="71" t="str">
+        <x:v>78D42383DA55AD7033DE4CAE4461FE2EF2EB4CE6BBFD1CA821522B2A0942CDA3</x:v>
+      </x:c>
+      <x:c r="H168" s="59" t="str">
+        <x:v>事务证据</x:v>
+      </x:c>
+      <x:c r="I168" s="69" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="J168" s="60" t="str">
+        <x:v>65/65真实WZL导出回读通过</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="169" ht="72" customHeight="1">
+      <x:c r="A169" s="58" t="str">
+        <x:v>EL-PARAM-MAT-WZX-HASH-BEFORE</x:v>
+      </x:c>
+      <x:c r="B169" s="59" t="str">
+        <x:v>材料图库</x:v>
+      </x:c>
+      <x:c r="C169" s="59" t="str">
+        <x:v>Items.wzx写前SHA256</x:v>
+      </x:c>
+      <x:c r="D169" s="59" t="str">
+        <x:v>SHA256</x:v>
+      </x:c>
+      <x:c r="E169" s="59"/>
+      <x:c r="F169" s="59"/>
+      <x:c r="G169" s="71" t="str">
+        <x:v>74A1B3B5F2E5CF5A099F9D6DC7FDF8207A71B834CA4AD2A17B9F00FC328729C3</x:v>
+      </x:c>
+      <x:c r="H169" s="59" t="str">
+        <x:v>事务证据</x:v>
+      </x:c>
+      <x:c r="I169" s="69" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="J169" s="60" t="str">
+        <x:v>图标事务XYMI-20260822-013718-C9646062</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="170" ht="72" customHeight="1">
+      <x:c r="A170" s="61" t="str">
+        <x:v>EL-PARAM-MAT-WZX-HASH-AFTER</x:v>
+      </x:c>
+      <x:c r="B170" s="62" t="str">
+        <x:v>材料图库</x:v>
+      </x:c>
+      <x:c r="C170" s="62" t="str">
+        <x:v>Items.wzx写后SHA256</x:v>
+      </x:c>
+      <x:c r="D170" s="62" t="str">
+        <x:v>SHA256</x:v>
+      </x:c>
+      <x:c r="E170" s="62"/>
+      <x:c r="F170" s="62"/>
+      <x:c r="G170" s="72" t="str">
+        <x:v>620BD07248317FAC18F466B0FB3C9470FF4DF1285FBE9AD0A4A3A139A5D3F3361</x:v>
+      </x:c>
+      <x:c r="H170" s="62" t="str">
+        <x:v>事务证据</x:v>
+      </x:c>
+      <x:c r="I170" s="70" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="J170" s="63" t="str">
+        <x:v>65/65真实WZL导出回读通过</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Archive complete material code database
</commit_message>
<xml_diff>
--- a/codex_tasks/艾尔登法环_第一二大陆_Codex施工包_20260821/项目档案/02_已确认规则与数值.xlsx
+++ b/codex_tasks/艾尔登法环_第一二大陆_Codex施工包_20260821/项目档案/02_已确认规则与数值.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="Rb9ea2fdae01741dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="已确认规则" sheetId="2" r:id="R32798b0da3a84dbc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数值参数" sheetId="3" r:id="R5aeb581a34694f47"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="装备索引" sheetId="4" r:id="R5a124bac72994097"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="怪物索引" sheetId="5" r:id="Rc4b803820fd748e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="地图索引" sheetId="6" r:id="R8c8aa133c91b4226"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="掉落索引" sheetId="7" r:id="R1045cd007bbd41f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R0f242321b22c4b45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="已确认规则" sheetId="2" r:id="Ra055690535284d5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数值参数" sheetId="3" r:id="R04dca31198904ef0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="装备索引" sheetId="4" r:id="Re2589b853bef4105"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="怪物索引" sheetId="5" r:id="R1dbb94276da049f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="地图索引" sheetId="6" r:id="Rff3795122eda47b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="掉落索引" sheetId="7" r:id="R39af54fb22194fa6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5712,16 +5712,16 @@
         <x:v>材料编码库与装备编码库分开长期维护；材料物品ID、数据库Idx、Items背包图标Looks及用途映射以材料库原件为准，两库不得合并、互推或只保存摘要。</x:v>
       </x:c>
       <x:c r="D209" s="59" t="str">
-        <x:v>已确认</x:v>
+        <x:v>已确认并接续</x:v>
       </x:c>
       <x:c r="E209" s="69" t="n">
         <x:v>46256</x:v>
       </x:c>
       <x:c r="F209" s="59" t="str">
-        <x:v>用户2026-08-22要求完整继承</x:v>
+        <x:v>材料编码数据库.xlsx＋批次A完整成果目录</x:v>
       </x:c>
       <x:c r="G209" s="60" t="str">
-        <x:v>材料只使用Items图库时仍须独立登记，不从装备来源编号反推</x:v>
+        <x:v>以材料主索引为新增、查重和占用的唯一入口</x:v>
       </x:c>
     </x:row>
     <x:row r="210" ht="44" customHeight="1">
@@ -5735,16 +5735,16 @@
         <x:v>65件材料事务：图标65/65，Items图库数量由6398变为6463，Looks 6398—6462；数据库65/65，Idx 907—971；972—983预留0行；793/794/802保持不变。材料未写DnItems或StateItem。</x:v>
       </x:c>
       <x:c r="D210" s="59" t="str">
-        <x:v>事务已确认，原件待接续</x:v>
+        <x:v>原件已接续／65条逐行验证通过</x:v>
       </x:c>
       <x:c r="E210" s="69" t="n">
         <x:v>46256</x:v>
       </x:c>
       <x:c r="F210" s="59" t="str">
-        <x:v>20260822_0235_65材料图标与正式入库.txt</x:v>
+        <x:v>material_import_phase_a.7z完整成果目录</x:v>
       </x:c>
       <x:c r="G210" s="60" t="str">
-        <x:v>Git d9f705fbe8da4a017038568f9f8d5cbd1b504748；XYMI-20260822-013718-C9646062；XYMD-20260822-014350-1C7690A1；新专项4项＋既有材料批量13项通过</x:v>
+        <x:v>行级交叉检查0错误；M2加载与游戏内背包显示仍待验收</x:v>
       </x:c>
     </x:row>
     <x:row r="211" ht="44" customHeight="1">
@@ -5755,19 +5755,19 @@
         <x:v>材料施工</x:v>
       </x:c>
       <x:c r="C211" s="59" t="str">
-        <x:v>在65条逐行材料数据库原件接续前，Idx 907—971及Items Looks 6398—6462按已占用冻结，Idx 972—983按预留冻结；不新增材料编号，不把事务摘要冒充完整材料库。</x:v>
+        <x:v>Idx 907—971及Items Looks 6398—6462以完整材料库原件确认为已占用，Idx 972—983为预留冻结段且占用0行。新增材料前必须查权威库并登记事务。</x:v>
       </x:c>
       <x:c r="D211" s="59" t="str">
-        <x:v>立即生效</x:v>
+        <x:v>原件已确认／占用与预留冻结继续生效</x:v>
       </x:c>
       <x:c r="E211" s="69" t="n">
         <x:v>46256</x:v>
       </x:c>
       <x:c r="F211" s="59" t="str">
-        <x:v>用户2026-08-22要求完整继承</x:v>
+        <x:v>材料编码数据库.xlsx＋跨库核验</x:v>
       </x:c>
       <x:c r="G211" s="60" t="str">
-        <x:v>同数字Looks段与装备资源库暂列原件级核验项，不在缺少WZL差异时擅自判冲突或改号</x:v>
+        <x:v>Items Looks 6398—6462与装备库同号候选存在65个确认重叠；本轮不改装备表，但暂停该段作为新装备来源编号</x:v>
       </x:c>
     </x:row>
     <x:row r="212" ht="44" customHeight="1">
@@ -5837,6 +5837,29 @@
       </x:c>
       <x:c r="G214" s="63" t="str">
         <x:v>逐大陆名称、代码、基础爆率、奖励及登记是否消耗实物待确认</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="215">
+      <x:c r="A215" t="str">
+        <x:v>EL-MAT-CODEDB-INHERIT-001</x:v>
+      </x:c>
+      <x:c r="B215" t="str">
+        <x:v>材料库接续</x:v>
+      </x:c>
+      <x:c r="C215" t="str">
+        <x:v>完整成果目录已接续：65件新增材料的逻辑ID、名称、大陆、类别、模板、StdMode、Shape、Looks、Color、基础字段、图标与回读哈希、事务号已纳入独立材料编码数据库；3件保护材料另行保留。</x:v>
+      </x:c>
+      <x:c r="D215" t="str">
+        <x:v>已完整接续</x:v>
+      </x:c>
+      <x:c r="E215" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="F215" t="str">
+        <x:v>material_import_phase_a.7z／材料编码数据库.xlsx</x:v>
+      </x:c>
+      <x:c r="G215" t="str">
+        <x:v>新材料Idx、名称、Looks、逻辑ID、源图哈希、回读哈希均重复0；逐行关系错误0</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -10628,13 +10651,13 @@
         <x:v>65</x:v>
       </x:c>
       <x:c r="H152" s="59" t="str">
-        <x:v>事务已确认，原件待接续</x:v>
+        <x:v>原件已接续并逐行验证</x:v>
       </x:c>
       <x:c r="I152" s="69" t="n">
         <x:v>46256</x:v>
       </x:c>
       <x:c r="J152" s="60" t="str">
-        <x:v>数据库事务XYMD-20260822-014350-1C7690A1</x:v>
+        <x:v>材料编码数据库.xlsx；数据库事务XYMD-20260822-014350-1C7690A1</x:v>
       </x:c>
     </x:row>
     <x:row r="153" ht="44" customHeight="1">
@@ -11183,6 +11206,194 @@
       </x:c>
       <x:c r="J170" s="63" t="str">
         <x:v>65/65真实WZL导出回读通过</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="171">
+      <x:c r="A171" t="str">
+        <x:v>EL-PARAM-MAT-CODEDB-ROWS</x:v>
+      </x:c>
+      <x:c r="B171" t="str">
+        <x:v>材料库</x:v>
+      </x:c>
+      <x:c r="C171" t="str">
+        <x:v>权威材料主索引总行数</x:v>
+      </x:c>
+      <x:c r="D171" t="str">
+        <x:v>条</x:v>
+      </x:c>
+      <x:c r="E171" t="n">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="F171" t="n">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="G171" t="n">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="H171" t="str">
+        <x:v>已核验</x:v>
+      </x:c>
+      <x:c r="I171" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="J171" t="str">
+        <x:v>3件保护材料＋65件新增材料</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="172">
+      <x:c r="A172" t="str">
+        <x:v>EL-PARAM-MAT-CODEDB-ROW-ERROR</x:v>
+      </x:c>
+      <x:c r="B172" t="str">
+        <x:v>质检</x:v>
+      </x:c>
+      <x:c r="C172" t="str">
+        <x:v>65件新增材料跨清单逐行关系错误</x:v>
+      </x:c>
+      <x:c r="D172" t="str">
+        <x:v>项</x:v>
+      </x:c>
+      <x:c r="E172" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F172" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G172" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H172" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="I172" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="J172" t="str">
+        <x:v>生成清单／图库回读／入库清单／已部署映射</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="173">
+      <x:c r="A173" t="str">
+        <x:v>EL-PARAM-MAT-ICON-FILES</x:v>
+      </x:c>
+      <x:c r="B173" t="str">
+        <x:v>质检</x:v>
+      </x:c>
+      <x:c r="C173" t="str">
+        <x:v>48×48 RGBA正式材料图标数</x:v>
+      </x:c>
+      <x:c r="D173" t="str">
+        <x:v>个</x:v>
+      </x:c>
+      <x:c r="E173" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="F173" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="G173" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="H173" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="I173" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="J173" t="str">
+        <x:v>icons/final实文件哈希与清单一致</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="174">
+      <x:c r="A174" t="str">
+        <x:v>EL-PARAM-MAT-CROSSDB-OVERLAP</x:v>
+      </x:c>
+      <x:c r="B174" t="str">
+        <x:v>跨库检查</x:v>
+      </x:c>
+      <x:c r="C174" t="str">
+        <x:v>材料Items Looks与装备库同号候选重叠</x:v>
+      </x:c>
+      <x:c r="D174" t="str">
+        <x:v>个</x:v>
+      </x:c>
+      <x:c r="E174" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="F174" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="G174" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="H174" t="str">
+        <x:v>已确认／装备候选暂停</x:v>
+      </x:c>
+      <x:c r="I174" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="J174" t="str">
+        <x:v>6398—6462全段重叠；本轮不改既有装备表</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="175">
+      <x:c r="A175" t="str">
+        <x:v>EL-PARAM-EQUIP-CANDIDATE-REMAIN</x:v>
+      </x:c>
+      <x:c r="B175" t="str">
+        <x:v>编码库</x:v>
+      </x:c>
+      <x:c r="C175" t="str">
+        <x:v>6396—7095候选段扣除材料Looks后的数字个数</x:v>
+      </x:c>
+      <x:c r="D175" t="str">
+        <x:v>个</x:v>
+      </x:c>
+      <x:c r="E175" t="n">
+        <x:v>635</x:v>
+      </x:c>
+      <x:c r="F175" t="n">
+        <x:v>635</x:v>
+      </x:c>
+      <x:c r="G175" t="n">
+        <x:v>635</x:v>
+      </x:c>
+      <x:c r="H175" t="str">
+        <x:v>仅候选／仍需实库查占用</x:v>
+      </x:c>
+      <x:c r="I175" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="J175" t="str">
+        <x:v>2个6396—6397＋633个6463—7095</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="176">
+      <x:c r="A176" t="str">
+        <x:v>EL-PARAM-MAT-PACKAGE-SHA256</x:v>
+      </x:c>
+      <x:c r="B176" t="str">
+        <x:v>证据</x:v>
+      </x:c>
+      <x:c r="C176" t="str">
+        <x:v>material_import_phase_a.7z SHA256</x:v>
+      </x:c>
+      <x:c r="D176" t="str">
+        <x:v>SHA256</x:v>
+      </x:c>
+      <x:c r="E176"/>
+      <x:c r="F176"/>
+      <x:c r="G176" t="str">
+        <x:v>7ece929bcdbad38efe68b7b34e7a6ea27b949292a2f2fab8d6ff575f75f29d88</x:v>
+      </x:c>
+      <x:c r="H176" t="str">
+        <x:v>已登记</x:v>
+      </x:c>
+      <x:c r="I176" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="J176" t="str">
+        <x:v>完整成果目录原包</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -12981,16 +13192,16 @@
         <x:v>Idx 907—971；Looks 6398—6462</x:v>
       </x:c>
       <x:c r="E14" s="62" t="str">
-        <x:v>实际材料库原件待从上个窗口完整成果目录接续</x:v>
+        <x:v>/传奇私服之旅/艾尔登法环项目档案/材料编码数据库.xlsx</x:v>
       </x:c>
       <x:c r="F14" s="70" t="n">
         <x:v>46256</x:v>
       </x:c>
       <x:c r="G14" s="62" t="str">
-        <x:v>972—983预留；793/794/802不变；只写Items图库</x:v>
+        <x:v>972—983预留；793/794/802不变；只写Items图库；6398—6462不得作为新装备Items来源编号</x:v>
       </x:c>
       <x:c r="H14" s="63" t="str">
-        <x:v>事务已确认，逐行原件缺失</x:v>
+        <x:v>原件已接续／65条逐行通过／游戏内待验收</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Sync core archives with C3-C10 framework
</commit_message>
<xml_diff>
--- a/codex_tasks/艾尔登法环_第一二大陆_Codex施工包_20260821/项目档案/02_已确认规则与数值.xlsx
+++ b/codex_tasks/艾尔登法环_第一二大陆_Codex施工包_20260821/项目档案/02_已确认规则与数值.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R0f242321b22c4b45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="已确认规则" sheetId="2" r:id="Ra055690535284d5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数值参数" sheetId="3" r:id="R04dca31198904ef0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="装备索引" sheetId="4" r:id="Re2589b853bef4105"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="怪物索引" sheetId="5" r:id="R1dbb94276da049f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="地图索引" sheetId="6" r:id="Rff3795122eda47b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="掉落索引" sheetId="7" r:id="R39af54fb22194fa6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R653ac072bb0b44a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="已确认规则" sheetId="2" r:id="Rb0a53c0427894aea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数值参数" sheetId="3" r:id="R5de56a3967c2496e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="装备索引" sheetId="4" r:id="Rb2692fbada684464"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="怪物索引" sheetId="5" r:id="R32640b05a2ae469d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="地图索引" sheetId="6" r:id="Rf2e5f13c0e4c40fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="掉落索引" sheetId="7" r:id="Ref021a6b8a244d96"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,12 +19,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="5">
+  <x:numFmts count="6">
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
     <x:numFmt numFmtId="201" formatCode="#,##0.00"/>
     <x:numFmt numFmtId="202" formatCode="0%"/>
     <x:numFmt numFmtId="203" formatCode="0.0%"/>
     <x:numFmt numFmtId="204" formatCode="0"/>
+    <x:numFmt numFmtId="205" formatCode="0.000000"/>
   </x:numFmts>
   <x:fonts count="8">
     <x:font>
@@ -69,7 +70,7 @@
       <x:name val="Microsoft YaHei"/>
     </x:font>
   </x:fonts>
-  <x:fills count="9">
+  <x:fills count="13">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -109,6 +110,26 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFE6F3EA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -253,7 +274,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="73">
+  <x:cellXfs count="115">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -434,6 +455,108 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="9" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="9" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="10" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="10" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="10" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="11" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="11" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="11" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="6" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="12" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="12" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="12" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -737,7 +860,7 @@
         <x:v>最高依据</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>最新明确确认 &gt; 本工作簿正式记录 &gt; 旧文件 &gt; 聊天记忆</x:v>
+        <x:v>最新明确确认／最新专题成品 &gt; 本工作簿正式记录 &gt; 旧文件 &gt; 聊天记忆</x:v>
       </x:c>
       <x:c r="C6"/>
       <x:c r="D6"/>
@@ -773,7 +896,7 @@
         <x:v>当前说明</x:v>
       </x:c>
       <x:c r="B9" s="30" t="str">
-        <x:v>现行范围为10个正式大陆＋3个预留主题；规则冲突按最新用户确认覆盖旧值，具体合成配方与成功率未确认时保持待定。</x:v>
+        <x:v>现行范围为10个正式大陆＋3个预留主题；功能与地图已冻结。NPC V0.2、命格100组、20转、六档攻速／TTK及第3—10大陆464怪／464专属来源框架按最新确认执行。</x:v>
       </x:c>
       <x:c r="C9"/>
       <x:c r="D9"/>
@@ -1523,19 +1646,19 @@
         <x:v>刀速</x:v>
       </x:c>
       <x:c r="C27" s="16" t="str">
-        <x:v>角色初始实际刀速约2刀/秒；第一大陆毕业实际刀速预计约3刀/秒。</x:v>
+        <x:v>攻速点与刀速必须分开：生效攻速点S_eff须先依六档实测关系换算成刀/秒，再进入DPS和TTK。旧“初始约2刀、一大陆毕业约3刀”只作历史约数。</x:v>
       </x:c>
       <x:c r="D27" s="23" t="str">
-        <x:v>已确认</x:v>
+        <x:v>已确认（替代旧值）</x:v>
       </x:c>
       <x:c r="E27" s="21" t="n">
-        <x:v>46235</x:v>
+        <x:v>46267</x:v>
       </x:c>
       <x:c r="F27" s="16" t="str">
-        <x:v>2026-08-01用户补充</x:v>
+        <x:v>20260830_0242_攻速六档实测与数学关系闭环.txt</x:v>
       </x:c>
       <x:c r="G27" s="16" t="str">
-        <x:v>实际刀速是DPS输入；装备攻击速度字段与刀/秒的映射仍需实测</x:v>
+        <x:v>S_eff=0/10/20/30/40/50对应1.75/2.20/2.90/4.30/8.50/14.30刀/秒；约3刀仅在S_eff≈20时成立</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="15" hidden="0" customHeight="1">
@@ -1546,19 +1669,19 @@
         <x:v>伤害构成</x:v>
       </x:c>
       <x:c r="C28" s="16" t="str">
-        <x:v>满暴击时，常规最终伤害=攻击力×打怪伤害×伤害系数×神力倍数×攻击伤害×暴击伤害。</x:v>
+        <x:v>满暴击时，常规最终伤害=攻击力×打怪伤害×伤害系数×神力倍数×攻击伤害×暴击总倍率。若暴伤字段是额外比例，须先与基础暴击倍率合成总倍率。</x:v>
       </x:c>
       <x:c r="D28" s="23" t="str">
-        <x:v>已确认</x:v>
+        <x:v>已确认（基础暴击倍率待引擎确认）</x:v>
       </x:c>
       <x:c r="E28" s="21" t="n">
-        <x:v>46235</x:v>
+        <x:v>46267</x:v>
       </x:c>
       <x:c r="F28" s="16" t="str">
-        <x:v>2026-08-01用户补充</x:v>
+        <x:v>用户TTK口径／现行乘区规则</x:v>
       </x:c>
       <x:c r="G28" s="16" t="str">
-        <x:v>固定切割和处决不并入该常规公式，必须单独建模</x:v>
+        <x:v>非满暴时必须使用暴击期望乘区，不得把暴伤无条件乘到每刀</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="15" hidden="0" customHeight="1">
@@ -1788,7 +1911,7 @@
         <x:v>2026-08-09用户确认</x:v>
       </x:c>
       <x:c r="G38" s="16" t="str">
-        <x:v>实际刀速与字段映射仍需实测；现有装备表中的固定幸运待清理</x:v>
+        <x:v>攻速字段依六档实测映射换算刀/秒；现有装备表中的固定幸运待清理</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="15" hidden="0" customHeight="1">
@@ -4191,19 +4314,19 @@
         <x:v>功能NPC</x:v>
       </x:c>
       <x:c r="C143" s="30" t="str">
-        <x:v>前两大陆功能NPC规划只涉及初始之地和宁姆格福；漂流群岛不部署任何功能性NPC。</x:v>
+        <x:v>漂流群岛新增命格NPC；技能和两类收集图鉴使用页面／命令，不设置独立NPC。宁姆格福新增战灰NPC及群攻生肖LV1配方。</x:v>
       </x:c>
       <x:c r="D143" s="30" t="str">
-        <x:v>已确认</x:v>
+        <x:v>已确认（替代旧值）</x:v>
       </x:c>
       <x:c r="E143" s="30" t="n">
-        <x:v>46250</x:v>
+        <x:v>46266</x:v>
       </x:c>
       <x:c r="F143" s="30" t="str">
-        <x:v>2026-08-16用户确认</x:v>
+        <x:v>2026-09-01用户最新确认</x:v>
       </x:c>
       <x:c r="G143" s="30" t="str">
-        <x:v>守关、传送、地图任务等地图NPC不属于本条范围</x:v>
+        <x:v>替代漂流群岛不部署任何功能性NPC的旧口径</x:v>
       </x:c>
     </x:row>
     <x:row r="144" ht="15" hidden="0" customHeight="1">
@@ -4559,19 +4682,19 @@
         <x:v>前期阶段</x:v>
       </x:c>
       <x:c r="C159" s="30" t="str">
-        <x:v>初始营地建立转生、两件特殊装备和长期称号；第一大陆纯PVE开荒且无额外成长NPC；宁姆格福开放深度培养。</x:v>
+        <x:v>初始营地保留两件特殊装备和长期称号；第一大陆新增命格NPC；宁姆格福开放深度培养、战灰和群攻生肖LV1；转生分布到第4／6／8／10大陆。</x:v>
       </x:c>
       <x:c r="D159" s="30" t="str">
-        <x:v>已确认</x:v>
+        <x:v>已确认（替代旧值）</x:v>
       </x:c>
       <x:c r="E159" s="30" t="n">
-        <x:v>46255</x:v>
+        <x:v>46266</x:v>
       </x:c>
       <x:c r="F159" s="30" t="str">
-        <x:v>前期系统交接</x:v>
+        <x:v>十大陆NPC V0.2／用户确认</x:v>
       </x:c>
       <x:c r="G159" s="30" t="str">
-        <x:v>贯穿系统纵向成长，后续大陆不复制整套旧系统</x:v>
+        <x:v>旧初始营地转生与第一大陆无成长NPC口径废止</x:v>
       </x:c>
     </x:row>
     <x:row r="160" ht="15" hidden="0" customHeight="1">
@@ -4582,19 +4705,19 @@
         <x:v>转生</x:v>
       </x:c>
       <x:c r="C160" s="30" t="str">
-        <x:v>共1—10转；前5转用小卢恩，后5转用大卢恩，核心收益为神力倍攻。</x:v>
+        <x:v>共20转：利耶尼亚海域1—5、盖利德6—10、巨人山顶11—15、王城罗德尔16—20；每处1名NPC、各5级。核心收益为神力倍攻。</x:v>
       </x:c>
       <x:c r="D160" s="30" t="str">
-        <x:v>已确认</x:v>
+        <x:v>已确认（分段成本待总账）</x:v>
       </x:c>
       <x:c r="E160" s="30" t="n">
-        <x:v>46255</x:v>
+        <x:v>46266</x:v>
       </x:c>
       <x:c r="F160" s="30" t="str">
-        <x:v>前期系统交接</x:v>
+        <x:v>十大陆NPC V0.2／用户确认</x:v>
       </x:c>
       <x:c r="G160" s="30" t="str">
-        <x:v>每转消耗与神力增量待资源总账确定</x:v>
+        <x:v>旧初始营地1—10转、固定消耗与每转神力0.05废止</x:v>
       </x:c>
     </x:row>
     <x:row r="161" ht="15" hidden="0" customHeight="1">
@@ -4881,19 +5004,19 @@
         <x:v>系统扩展</x:v>
       </x:c>
       <x:c r="C173" s="30" t="str">
-        <x:v>后续大陆优先增加新玩法维度；贯穿系统纵向成长，禁止每大陆复制新转生、新锻体、新洗练、新称号。</x:v>
+        <x:v>当前版本停止新增功能，地图保持现状；后续只落地既有NPC、怪物、爆率、装备、材料、货币及其数值平衡。</x:v>
       </x:c>
       <x:c r="D173" s="30" t="str">
-        <x:v>已确认</x:v>
+        <x:v>已确认（替代旧扩展口径）</x:v>
       </x:c>
       <x:c r="E173" s="30" t="n">
-        <x:v>46255</x:v>
+        <x:v>46266</x:v>
       </x:c>
       <x:c r="F173" s="30" t="str">
-        <x:v>前期系统交接</x:v>
+        <x:v>2026-09-01用户确认</x:v>
       </x:c>
       <x:c r="G173" s="30" t="str">
-        <x:v>控制系统膨胀</x:v>
+        <x:v>现有命格、战灰、群攻生肖和20转属于已确认既有功能</x:v>
       </x:c>
     </x:row>
     <x:row r="174" ht="15" hidden="0" customHeight="1">
@@ -5801,16 +5924,16 @@
         <x:v>收集图鉴</x:v>
       </x:c>
       <x:c r="C213" s="59" t="str">
-        <x:v>专属装备收集图鉴由命令触发脚本处理，不设置独立NPC；当前窗口提供单件收集奖励及大陆全部装备收集奖励表。</x:v>
+        <x:v>专属装备收集图鉴由命令触发脚本处理，不设置独立NPC；登记时消耗对应装备1件且不收金币、元宝或灵符。当前窗口提供单件及大陆全收集奖励表。</x:v>
       </x:c>
       <x:c r="D213" s="59" t="str">
-        <x:v>结构已确认，数值待定</x:v>
+        <x:v>结构与消耗已确认，数值待定</x:v>
       </x:c>
       <x:c r="E213" s="69" t="n">
-        <x:v>46256</x:v>
+        <x:v>46266</x:v>
       </x:c>
       <x:c r="F213" s="59" t="str">
-        <x:v>用户2026-08-22最新澄清</x:v>
+        <x:v>NPC V0.2／用户确认</x:v>
       </x:c>
       <x:c r="G213" s="60" t="str">
         <x:v>逐件奖励、页面划分和整页处决未确认时不得猜填</x:v>
@@ -5824,19 +5947,19 @@
         <x:v>收集图鉴</x:v>
       </x:c>
       <x:c r="C214" s="62" t="str">
-        <x:v>每个正式大陆另设1件不可装备、可收集的大陆专属图鉴材料，由本大陆所有怪物掉落；收集价值和奖励强度高于普通单件专属。</x:v>
+        <x:v>每个正式大陆另设1件不可装备、可收集的大陆专属图鉴材料，由本大陆所有怪物掉落；登记时消耗实物1件且不收金币、元宝或灵符。</x:v>
       </x:c>
       <x:c r="D214" s="62" t="str">
-        <x:v>结构已确认，细项待定</x:v>
+        <x:v>结构与消耗已确认，细项待定</x:v>
       </x:c>
       <x:c r="E214" s="70" t="n">
-        <x:v>46256</x:v>
+        <x:v>46266</x:v>
       </x:c>
       <x:c r="F214" s="62" t="str">
-        <x:v>用户2026-08-22新增</x:v>
+        <x:v>NPC V0.2／用户确认</x:v>
       </x:c>
       <x:c r="G214" s="63" t="str">
-        <x:v>逐大陆名称、代码、基础爆率、奖励及登记是否消耗实物待确认</x:v>
+        <x:v>逐大陆名称、代码、基础爆率和奖励待确认</x:v>
       </x:c>
     </x:row>
     <x:row r="215">
@@ -5860,6 +5983,742 @@
       </x:c>
       <x:c r="G215" t="str">
         <x:v>新材料Idx、名称、Looks、逻辑ID、源图哈希、回读哈希均重复0；逐行关系错误0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="216" ht="34" customHeight="1">
+      <x:c r="A216" s="82" t="str">
+        <x:v>EL-LINK-AUDIT-001</x:v>
+      </x:c>
+      <x:c r="B216" s="83" t="str">
+        <x:v>档案依据</x:v>
+      </x:c>
+      <x:c r="C216" s="83" t="str">
+        <x:v>外部ChatGPT共享链接和旧对话只用于查漏补缺；现行规则仍以用户最新确认、最新专题成品和六份核心档案为准。</x:v>
+      </x:c>
+      <x:c r="D216" s="91" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="E216" s="94" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="F216" s="83" t="str">
+        <x:v>2026-09-01用户确认</x:v>
+      </x:c>
+      <x:c r="G216" s="84" t="str">
+        <x:v>未重新确认的旧想法不得回填</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="217" ht="34" customHeight="1">
+      <x:c r="A217" s="85" t="str">
+        <x:v>EL-FEATURE-FREEZE-001</x:v>
+      </x:c>
+      <x:c r="B217" s="86" t="str">
+        <x:v>施工边界</x:v>
+      </x:c>
+      <x:c r="C217" s="86" t="str">
+        <x:v>当前版本不再新增功能，地图已经完成且不再修改；后续只落地NPC、怪物、爆率、装备、材料、货币及平衡。</x:v>
+      </x:c>
+      <x:c r="D217" s="92" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="E217" s="95" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="F217" s="86" t="str">
+        <x:v>2026-09-01用户确认</x:v>
+      </x:c>
+      <x:c r="G217" s="87" t="str">
+        <x:v>禁止恢复旧扩展功能</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="218" ht="34" customHeight="1">
+      <x:c r="A218" s="85" t="str">
+        <x:v>EL-ARCHIVE-PERIODIC-001</x:v>
+      </x:c>
+      <x:c r="B218" s="86" t="str">
+        <x:v>归档制度</x:v>
+      </x:c>
+      <x:c r="C218" s="86" t="str">
+        <x:v>长对话每积累一批实质确认或接近上下文切换时，主动总结并同步六份核心档案。</x:v>
+      </x:c>
+      <x:c r="D218" s="92" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="E218" s="95" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="F218" s="86" t="str">
+        <x:v>2026-09-01用户要求</x:v>
+      </x:c>
+      <x:c r="G218" s="87" t="str">
+        <x:v>不得只依赖聊天窗口记忆</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="219" ht="34" customHeight="1">
+      <x:c r="A219" s="85" t="str">
+        <x:v>EL-FATE-SYSTEM-001</x:v>
+      </x:c>
+      <x:c r="B219" s="86" t="str">
+        <x:v>命格</x:v>
+      </x:c>
+      <x:c r="C219" s="86" t="str">
+        <x:v>命格暂用灵玉位置，是最多8槽的逐槽独立高级洗练；一次只重洗当前第X槽，各槽保底独立。</x:v>
+      </x:c>
+      <x:c r="D219" s="92" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="E219" s="95" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="F219" s="86" t="str">
+        <x:v>命格界面／用户确认</x:v>
+      </x:c>
+      <x:c r="G219" s="87" t="str">
+        <x:v>脚本与界面已完成，当前窗口不重做</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="220" ht="34" customHeight="1">
+      <x:c r="A220" s="85" t="str">
+        <x:v>EL-FATE-PITY-001</x:v>
+      </x:c>
+      <x:c r="B220" s="86" t="str">
+        <x:v>命格</x:v>
+      </x:c>
+      <x:c r="C220" s="86" t="str">
+        <x:v>命格保底沿用现有界面：20次必出红色、每10次参与彩色判定、100次必出彩色。</x:v>
+      </x:c>
+      <x:c r="D220" s="92" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="E220" s="95" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="F220" s="86" t="str">
+        <x:v>命格界面／用户确认</x:v>
+      </x:c>
+      <x:c r="G220" s="87" t="str">
+        <x:v>所有保底均按当前选择槽独立计算</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="221" ht="34" customHeight="1">
+      <x:c r="A221" s="85" t="str">
+        <x:v>EL-FATE-TIER-001</x:v>
+      </x:c>
+      <x:c r="B221" s="86" t="str">
+        <x:v>命格</x:v>
+      </x:c>
+      <x:c r="C221" s="86" t="str">
+        <x:v>绿、黄、橙、红、彩各20个，共100组；强度约1／2／3／4／6，彩色明显优于红色。橙色起可出现受控稀有词条，彩色最多3条。</x:v>
+      </x:c>
+      <x:c r="D221" s="92" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="E221" s="95" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="F221" s="86" t="str">
+        <x:v>41_命格内容与多色属性.xlsx／用户确认</x:v>
+      </x:c>
+      <x:c r="G221" s="87" t="str">
+        <x:v>红色与彩色稀有词条数不固定，按实战强度控制</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="222" ht="34" customHeight="1">
+      <x:c r="A222" s="85" t="str">
+        <x:v>EL-FATE-RARE-001</x:v>
+      </x:c>
+      <x:c r="B222" s="86" t="str">
+        <x:v>命格</x:v>
+      </x:c>
+      <x:c r="C222" s="86" t="str">
+        <x:v>受控稀有词条：伤害系数、最大爆率、首尾斩杀、处决倍率、处决时间、处决、吸血、伤害吸收上限、人物爆率（元素爆率）、攻击速度、攻速突破。</x:v>
+      </x:c>
+      <x:c r="D222" s="92" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="E222" s="95" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="F222" s="86" t="str">
+        <x:v>用户命格属性确认</x:v>
+      </x:c>
+      <x:c r="G222" s="87" t="str">
+        <x:v>必须计入全服总预算</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="223" ht="34" customHeight="1">
+      <x:c r="A223" s="85" t="str">
+        <x:v>EL-FATE-ECON-001</x:v>
+      </x:c>
+      <x:c r="B223" s="86" t="str">
+        <x:v>命格</x:v>
+      </x:c>
+      <x:c r="C223" s="86" t="str">
+        <x:v>命格材料所有大陆略低爆率掉落，并可用灵符购买；自然产出支持普通洗练但不足以稳定全身彩色，全彩为明显付费追求。</x:v>
+      </x:c>
+      <x:c r="D223" s="92" t="str">
+        <x:v>已确认（数量待总账）</x:v>
+      </x:c>
+      <x:c r="E223" s="95" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="F223" s="86" t="str">
+        <x:v>用户付费定位确认</x:v>
+      </x:c>
+      <x:c r="G223" s="87" t="str">
+        <x:v>不直接出售红色或彩色结果</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="224" ht="34" customHeight="1">
+      <x:c r="A224" s="85" t="str">
+        <x:v>EL-ATKSPEED-BREAK-001</x:v>
+      </x:c>
+      <x:c r="B224" s="86" t="str">
+        <x:v>攻速突破</x:v>
+      </x:c>
+      <x:c r="C224" s="86" t="str">
+        <x:v>生效攻速点S_eff=min(装备攻速,20+攻速突破)。普通上限20，突破技术上限30，S_eff理论上限50；刀速须再通过实测映射换算。</x:v>
+      </x:c>
+      <x:c r="D224" s="92" t="str">
+        <x:v>已确认（总投放受控）</x:v>
+      </x:c>
+      <x:c r="E224" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="F224" s="86" t="str">
+        <x:v>2026-09-02用户补充／六档攻速实测</x:v>
+      </x:c>
+      <x:c r="G224" s="87" t="str">
+        <x:v>普攻DPS/TTK顶级稀有属性；现版本全程约20点，命格3—5点，单把武器最高5点</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="225" ht="34" customHeight="1">
+      <x:c r="A225" s="85" t="str">
+        <x:v>EL-NPC-V02-001</x:v>
+      </x:c>
+      <x:c r="B225" s="86" t="str">
+        <x:v>NPC规划</x:v>
+      </x:c>
+      <x:c r="C225" s="86" t="str">
+        <x:v>第1—10大陆均保留合成NPC；第3、5、7、9大陆各2名，第10大陆3名，其余大陆1名。命格、战灰、转生、群攻生肖升级等系统NPC另计。</x:v>
+      </x:c>
+      <x:c r="D225" s="92" t="str">
+        <x:v>结构已确认，数值待定</x:v>
+      </x:c>
+      <x:c r="E225" s="95" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="F225" s="86" t="str">
+        <x:v>20260831_十大陆NPC规划大框_假设占位版.md</x:v>
+      </x:c>
+      <x:c r="G225" s="87" t="str">
+        <x:v>金币元宝交叉使用；产物可覆盖装备、时装、生肖、首饰盒和称号</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="226" ht="34" customHeight="1">
+      <x:c r="A226" s="85" t="str">
+        <x:v>EL-AOE-ZODIAC-001</x:v>
+      </x:c>
+      <x:c r="B226" s="86" t="str">
+        <x:v>群攻生肖</x:v>
+      </x:c>
+      <x:c r="C226" s="86" t="str">
+        <x:v>宁姆格福合成LV1：2×2范围、2秒一次、自身攻击力伤害；第3、5、7、9大陆依次升级，最终LV5为3×3范围、1秒。</x:v>
+      </x:c>
+      <x:c r="D226" s="92" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="E226" s="95" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="F226" s="86" t="str">
+        <x:v>NPC V0.2／用户确认</x:v>
+      </x:c>
+      <x:c r="G226" s="87" t="str">
+        <x:v>主要为观赏与清怪反馈，不计入主线标准DPS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="227" ht="34" customHeight="1">
+      <x:c r="A227" s="88" t="str">
+        <x:v>EL-NPC-CURRENCY-CROSS-001</x:v>
+      </x:c>
+      <x:c r="B227" s="89" t="str">
+        <x:v>货币</x:v>
+      </x:c>
+      <x:c r="C227" s="89" t="str">
+        <x:v>金币与元宝无高低级关系；配方可单用金币、单用元宝或同时使用，并在相邻大陆交替制造币种缺口。</x:v>
+      </x:c>
+      <x:c r="D227" s="93" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="E227" s="96" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="F227" s="89" t="str">
+        <x:v>NPC V0.2／用户确认</x:v>
+      </x:c>
+      <x:c r="G227" s="90" t="str">
+        <x:v>阶段自产30%—40%，市场补足60%—70%</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="228" ht="38" customHeight="1">
+      <x:c r="A228" s="82" t="str">
+        <x:v>EL-DROP-BOSS-MAP-EXCLUSIVE-001</x:v>
+      </x:c>
+      <x:c r="B228" s="83" t="str">
+        <x:v>怪物掉落</x:v>
+      </x:c>
+      <x:c r="C228" s="83" t="str">
+        <x:v>常规BOSS除自身专属外，还可兼掉所在地图的小怪专属；BOSS自身专属池、本地图小怪专属兼掉池与每日额外守关BOSS福利池必须分开配置、分开核算。</x:v>
+      </x:c>
+      <x:c r="D228" s="97" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="E228" s="94" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="F228" s="83" t="str">
+        <x:v>2026-09-02用户确认</x:v>
+      </x:c>
+      <x:c r="G228" s="84" t="str">
+        <x:v>禁止把同一产出重复计入基础掉落与每日福利</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="229" ht="38" customHeight="1">
+      <x:c r="A229" s="85" t="str">
+        <x:v>EL-EQUIP-SAMENAME-FIXED-001</x:v>
+      </x:c>
+      <x:c r="B229" s="86" t="str">
+        <x:v>装备基础</x:v>
+      </x:c>
+      <x:c r="C229" s="86" t="str">
+        <x:v>同名装备的基础数据库属性固定一致；同一个名称不得制作基础属性高低不同的随机版本，个体差异只来自既有鉴定和洗练。</x:v>
+      </x:c>
+      <x:c r="D229" s="98" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="E229" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="F229" s="86" t="str">
+        <x:v>2026-09-02用户确认</x:v>
+      </x:c>
+      <x:c r="G229" s="87" t="str">
+        <x:v>不同名称装备仍可采用多路线设计</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="230" ht="38" customHeight="1">
+      <x:c r="A230" s="85" t="str">
+        <x:v>EL-EXCLUSIVE-DUP-SINK-001</x:v>
+      </x:c>
+      <x:c r="B230" s="86" t="str">
+        <x:v>专属消耗</x:v>
+      </x:c>
+      <x:c r="C230" s="86" t="str">
+        <x:v>重复专属用于任务提交、称号成长或分解；后续资源总账逐项确定对应消耗端、需求数量和产物。</x:v>
+      </x:c>
+      <x:c r="D230" s="98" t="str">
+        <x:v>已确认（细项待总账）</x:v>
+      </x:c>
+      <x:c r="E230" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="F230" s="86" t="str">
+        <x:v>2026-09-02用户确认</x:v>
+      </x:c>
+      <x:c r="G230" s="87" t="str">
+        <x:v>未明确前不得将同一件重复计入多个消耗端</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="231" ht="38" customHeight="1">
+      <x:c r="A231" s="88" t="str">
+        <x:v>EL-EXISTING-OUTSCOPE-001</x:v>
+      </x:c>
+      <x:c r="B231" s="89" t="str">
+        <x:v>施工边界</x:v>
+      </x:c>
+      <x:c r="C231" s="89" t="str">
+        <x:v>全服唯一首杀／首爆、极稀有装备自动进入背包、必要战士辅助技能及少量指定PK区域均为本服既有机制，但不属于当前窗口的数据设计职责。</x:v>
+      </x:c>
+      <x:c r="D231" s="99" t="str">
+        <x:v>既有系统／职责外</x:v>
+      </x:c>
+      <x:c r="E231" s="96" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="F231" s="89" t="str">
+        <x:v>2026-09-02用户确认</x:v>
+      </x:c>
+      <x:c r="G231" s="90" t="str">
+        <x:v>只记录边界，不重做脚本、技能或PK区域</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="232" ht="44" customHeight="1">
+      <x:c r="A232" s="82" t="str">
+        <x:v>EL-ATKSPEED-MEASURED-001</x:v>
+      </x:c>
+      <x:c r="B232" s="83" t="str">
+        <x:v>攻速实测</x:v>
+      </x:c>
+      <x:c r="C232" s="83" t="str">
+        <x:v>生效攻速点S_eff=0/10/20/30/40/50的实测刀速为1.75/2.20/2.90/4.30/8.50/14.30刀/秒，实测刀间隔为571.429/454.545/344.828/232.558/117.647/69.930ms。</x:v>
+      </x:c>
+      <x:c r="D232" s="100" t="str">
+        <x:v>已实测</x:v>
+      </x:c>
+      <x:c r="E232" s="94" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="F232" s="83" t="str">
+        <x:v>20260830_0242_攻速六档实测与数学关系闭环.txt</x:v>
+      </x:c>
+      <x:c r="G232" s="84" t="str">
+        <x:v>普通高HP目标的10秒[@Attack]计数；不用训练假人/全MISS目标</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="233" ht="44" customHeight="1">
+      <x:c r="A233" s="85" t="str">
+        <x:v>EL-ATKSPEED-FIT-001</x:v>
+      </x:c>
+      <x:c r="B233" s="86" t="str">
+        <x:v>攻速公式</x:v>
+      </x:c>
+      <x:c r="C233" s="86" t="str">
+        <x:v>S_eff=0—40时，实测刀间隔T(ms)=570.111430-11.295503×S_eff，R²=0.99991317，刀速v=1000/T。</x:v>
+      </x:c>
+      <x:c r="D233" s="101" t="str">
+        <x:v>已实测</x:v>
+      </x:c>
+      <x:c r="E233" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="F233" s="86" t="str">
+        <x:v>20260830_0242_攻速六档实测与数学关系闭环.txt</x:v>
+      </x:c>
+      <x:c r="G233" s="87" t="str">
+        <x:v>仅用0—40；不得直线外推到50</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="234" ht="44" customHeight="1">
+      <x:c r="A234" s="85" t="str">
+        <x:v>EL-ATKSPEED-EVIDENCE-BOUNDARY-001</x:v>
+      </x:c>
+      <x:c r="B234" s="86" t="str">
+        <x:v>攻速边界</x:v>
+      </x:c>
+      <x:c r="C234" s="86" t="str">
+        <x:v>S_eff=50的69.930ms/14.30刀每秒是独立实测点；41—49档尚未逐档实测，且该单点不证明引擎天然硬上限。</x:v>
+      </x:c>
+      <x:c r="D234" s="101" t="str">
+        <x:v>边界已确认</x:v>
+      </x:c>
+      <x:c r="E234" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="F234" s="86" t="str">
+        <x:v>20260830_0242_攻速六档实测与数学关系闭环.txt</x:v>
+      </x:c>
+      <x:c r="G234" s="87" t="str">
+        <x:v>max(69.930,570.111430-11.295503×S_eff)只作0—50业务预算候选模型</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="235" ht="44" customHeight="1">
+      <x:c r="A235" s="85" t="str">
+        <x:v>EL-CRIT-EV-001</x:v>
+      </x:c>
+      <x:c r="B235" s="86" t="str">
+        <x:v>暴击期望</x:v>
+      </x:c>
+      <x:c r="C235" s="86" t="str">
+        <x:v>暴击率p、暴击总倍率M时，暴击期望乘区=(1-p)+p×M=1+p×(M-1)。若暴伤字段为额外比例b，则M=基础暴击倍率+b。</x:v>
+      </x:c>
+      <x:c r="D235" s="101" t="str">
+        <x:v>公式已确认，基础倍率待引擎确认</x:v>
+      </x:c>
+      <x:c r="E235" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="F235" s="86" t="str">
+        <x:v>2026-09-02用户TTK口径</x:v>
+      </x:c>
+      <x:c r="G235" s="87" t="str">
+        <x:v>满暴公式只是p=100%特例；命中率、目标暴击抗性存在时另行计入p</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="236" ht="44" customHeight="1">
+      <x:c r="A236" s="85" t="str">
+        <x:v>EL-DPS-TTK-CALC-001</x:v>
+      </x:c>
+      <x:c r="B236" s="86" t="str">
+        <x:v>DPS/TTK</x:v>
+      </x:c>
+      <x:c r="C236" s="86" t="str">
+        <x:v>先按攻击力×各已确认乘区、怪物防御/减免和概率期望计算单刀期望伤害；再乘实测刀速得DPS。净DPS扣除怪物回复，连续近似TTK=怪物HP/净DPS。</x:v>
+      </x:c>
+      <x:c r="D236" s="101" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="E236" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="F236" s="86" t="str">
+        <x:v>2026-09-02用户确认</x:v>
+      </x:c>
+      <x:c r="G236" s="87" t="str">
+        <x:v>理论计算在前，进服用于校准；15%不再是全服统一硬门槛，重点排除无法推进、单属性失控和明显结算错误</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="237" ht="44" customHeight="1">
+      <x:c r="A237" s="85" t="str">
+        <x:v>EL-DPS-TTK-DISCRETE-001</x:v>
+      </x:c>
+      <x:c r="B237" s="86" t="str">
+        <x:v>DPS/TTK</x:v>
+      </x:c>
+      <x:c r="C237" s="86" t="str">
+        <x:v>固定切割、首尾斩杀、处决窗口、周期伤害和低刀数目标不并入单一常规乘区，必须单列或逐刀模拟。</x:v>
+      </x:c>
+      <x:c r="D237" s="101" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="E237" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="F237" s="86" t="str">
+        <x:v>现行乘区规则/用户TTK口径</x:v>
+      </x:c>
+      <x:c r="G237" s="87" t="str">
+        <x:v>普攻与技能动作/CD不得默认使用同一攻速倍率</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="238" ht="44" customHeight="1">
+      <x:c r="A238" s="88" t="str">
+        <x:v>EL-ATKSPEED-BUDGET-001</x:v>
+      </x:c>
+      <x:c r="B238" s="89" t="str">
+        <x:v>攻速突破</x:v>
+      </x:c>
+      <x:c r="C238" s="89" t="str">
+        <x:v>攻速突破是对普通攻击DPS/TTK提升最高的顶级稀有属性之一。现版本全游戏合计约投放20点；命格渠道合计3—5点，单把武器按稀有度最高5点。</x:v>
+      </x:c>
+      <x:c r="D238" s="102" t="str">
+        <x:v>已确认（其余渠道待分配）</x:v>
+      </x:c>
+      <x:c r="E238" s="96" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="F238" s="89" t="str">
+        <x:v>2026-09-02用户补充</x:v>
+      </x:c>
+      <x:c r="G238" s="90" t="str">
+        <x:v>突破技术上限30只是上限，不等于现版本投放30点</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="239" ht="46" customHeight="1">
+      <x:c r="A239" s="82" t="str">
+        <x:v>EL-C3C10-MONSTER-FRAME-001</x:v>
+      </x:c>
+      <x:c r="B239" s="83" t="str">
+        <x:v>怪物结构</x:v>
+      </x:c>
+      <x:c r="C239" s="83" t="str">
+        <x:v>第3—10大陆38组、144图共464怪：普通228、稀有152、地图BOSS 76、大陆最终BOSS 8；每组6普通、4稀有、2地图BOSS，每大陆最终地图另设1只最终BOSS。</x:v>
+      </x:c>
+      <x:c r="D239" s="105" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="E239" s="94" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="F239" s="83" t="str">
+        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.0.xlsx</x:v>
+      </x:c>
+      <x:c r="G239" s="84" t="str">
+        <x:v>每只怪均已绑定准确地图号与地图名</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="240" ht="46" customHeight="1">
+      <x:c r="A240" s="85" t="str">
+        <x:v>EL-C3C10-EXCLUSIVE-001</x:v>
+      </x:c>
+      <x:c r="B240" s="86" t="str">
+        <x:v>专属结构</x:v>
+      </x:c>
+      <x:c r="C240" s="86" t="str">
+        <x:v>464只怪物分别绑定464件唯一专属；普通定向专属只用武器、衣服、头盔、项链、手镯、戒指、腰带、鞋子、斗笠、盾牌、勋章11栏位。</x:v>
+      </x:c>
+      <x:c r="D240" s="106" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="E240" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="F240" s="86" t="str">
+        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.0.xlsx</x:v>
+      </x:c>
+      <x:c r="G240" s="87" t="str">
+        <x:v>马牌、战鼓/军鼓、灵玉、宝石禁用；生肖不参与；六个时装首饰盒保留给追梦神器</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="241" ht="46" customHeight="1">
+      <x:c r="A241" s="85" t="str">
+        <x:v>EL-C3C10-DROP-POOLS-001</x:v>
+      </x:c>
+      <x:c r="B241" s="86" t="str">
+        <x:v>掉落结构</x:v>
+      </x:c>
+      <x:c r="C241" s="86" t="str">
+        <x:v>怪物自身专属、常规BOSS兼掉、本大陆既有材料、大陆收藏材料、追梦神器公共奖池分别配置、分别核算。</x:v>
+      </x:c>
+      <x:c r="D241" s="106" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="E241" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="F241" s="86" t="str">
+        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.0.xlsx</x:v>
+      </x:c>
+      <x:c r="G241" s="87" t="str">
+        <x:v>不得将BOSS兼掉与每日守关福利池重复计账</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="242" ht="46" customHeight="1">
+      <x:c r="A242" s="85" t="str">
+        <x:v>EL-C3C10-MATERIAL-001</x:v>
+      </x:c>
+      <x:c r="B242" s="86" t="str">
+        <x:v>材料来源</x:v>
+      </x:c>
+      <x:c r="C242" s="86" t="str">
+        <x:v>第3—10大陆沿用56件已入库材料，每大陆7件，锁定Idx 916—971、Items Looks 6407—6462；本轮只建立来源关系。</x:v>
+      </x:c>
+      <x:c r="D242" s="106" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="E242" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="F242" s="86" t="str">
+        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.0.xlsx</x:v>
+      </x:c>
+      <x:c r="G242" s="87" t="str">
+        <x:v>冻结预留Idx 972—983不得直接启用</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="243" ht="46" customHeight="1">
+      <x:c r="A243" s="85" t="str">
+        <x:v>EL-C3C10-COLLECTIBLE-001</x:v>
+      </x:c>
+      <x:c r="B243" s="86" t="str">
+        <x:v>大陆图鉴</x:v>
+      </x:c>
+      <x:c r="C243" s="86" t="str">
+        <x:v>第3—10大陆8件收藏材料名称定稿：西境风痕碑拓、月潮忆珀、湖心月谱残章、熔原罪火残章、永霜朝圣痕、穹霜碑珀、古坛鎏叶髓、穹律鎏痕拓片。</x:v>
+      </x:c>
+      <x:c r="D243" s="106" t="str">
+        <x:v>名称已确认</x:v>
+      </x:c>
+      <x:c r="E243" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="F243" s="86" t="str">
+        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.0.xlsx</x:v>
+      </x:c>
+      <x:c r="G243" s="87" t="str">
+        <x:v>材料代码、基础爆率和登记奖励待资源总账</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="244" ht="46" customHeight="1">
+      <x:c r="A244" s="85" t="str">
+        <x:v>EL-MAP-MOONWATER-001</x:v>
+      </x:c>
+      <x:c r="B244" s="86" t="str">
+        <x:v>地图命名</x:v>
+      </x:c>
+      <x:c r="C244" s="86" t="str">
+        <x:v>正式名称为雾月水庭，不是雾月水宫；地图链为XX338→XX339→XX331。</x:v>
+      </x:c>
+      <x:c r="D244" s="106" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="E244" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="F244" s="86" t="str">
+        <x:v>2026-09-02用户确认</x:v>
+      </x:c>
+      <x:c r="G244" s="87" t="str">
+        <x:v>旧记录中的雾月水宫仅保留为历史转录</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="245" ht="46" customHeight="1">
+      <x:c r="A245" s="85" t="str">
+        <x:v>EL-C3-SLOT-FIX-001</x:v>
+      </x:c>
+      <x:c r="B245" s="86" t="str">
+        <x:v>专属纠错</x:v>
+      </x:c>
+      <x:c r="C245" s="86" t="str">
+        <x:v>第3大陆4件误占灵玉栏位的专属改为霆崖祭冠/头盔、黯幕咒戒/戒指、幽坛引魂铃/项链、赐光祷誓镯/手镯。</x:v>
+      </x:c>
+      <x:c r="D245" s="106" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="E245" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="F245" s="86" t="str">
+        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.0.xlsx</x:v>
+      </x:c>
+      <x:c r="G245" s="87" t="str">
+        <x:v>灵玉继续保留给命格系统</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="246" ht="46" customHeight="1">
+      <x:c r="A246" s="85" t="str">
+        <x:v>EL-TTK-TOLERANCE-001</x:v>
+      </x:c>
+      <x:c r="B246" s="86" t="str">
+        <x:v>验算边界</x:v>
+      </x:c>
+      <x:c r="C246" s="86" t="str">
+        <x:v>DPS/TTK偏差不超过15%不再作为全服通用硬门槛；允许流派、养成与攻速突破造成数倍效率差。</x:v>
+      </x:c>
+      <x:c r="D246" s="106" t="str">
+        <x:v>已确认（替代旧硬门槛）</x:v>
+      </x:c>
+      <x:c r="E246" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="F246" s="86" t="str">
+        <x:v>2026-09-02用户确认</x:v>
+      </x:c>
+      <x:c r="G246" s="87" t="str">
+        <x:v>理论与实测仍用于排除无法推进、单属性失控及明显结算错误</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="247" ht="46" customHeight="1">
+      <x:c r="A247" s="88" t="str">
+        <x:v>EL-SHOP-FATE-MATERIAL-001</x:v>
+      </x:c>
+      <x:c r="B247" s="89" t="str">
+        <x:v>商店例外</x:v>
+      </x:c>
+      <x:c r="C247" s="89" t="str">
+        <x:v>商店不出售常规材料的原则保留；命格洗练材料可用灵符购买，是已确认例外。</x:v>
+      </x:c>
+      <x:c r="D247" s="107" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="E247" s="96" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="F247" s="89" t="str">
+        <x:v>命格系统最终口径</x:v>
+      </x:c>
+      <x:c r="G247" s="90" t="str">
+        <x:v>自然掉落不足以支持全彩，全彩属于付费追求</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6389,13 +7248,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="H18" s="23" t="str">
-        <x:v>已确认</x:v>
+        <x:v>历史约数／已被实测替代</x:v>
       </x:c>
       <x:c r="I18" s="21" t="n">
-        <x:v>46235</x:v>
+        <x:v>46267</x:v>
       </x:c>
       <x:c r="J18" s="16" t="str">
-        <x:v>不是装备攻击速度字段</x:v>
+        <x:v>不得作为攻速字段映射；S_eff=0的正式实测为1.75刀/秒</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
@@ -6421,13 +7280,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="H19" s="23" t="str">
-        <x:v>已确认</x:v>
+        <x:v>历史约数／有条件成立</x:v>
       </x:c>
       <x:c r="I19" s="21" t="n">
-        <x:v>46235</x:v>
+        <x:v>46267</x:v>
       </x:c>
       <x:c r="J19" s="16" t="str">
-        <x:v>约值；用于最终DPS模型</x:v>
+        <x:v>只在角色S_eff≈20时约等于2.9刀/秒；阶段快照必须先确认S_eff</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
@@ -6519,7 +7378,7 @@
         <x:v>46235</x:v>
       </x:c>
       <x:c r="J22" s="16" t="str">
-        <x:v>与实际刀/秒映射待实测</x:v>
+        <x:v>攻速字段依六档实测关系换算为刀/秒</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
@@ -11196,16 +12055,16 @@
       <x:c r="E170" s="62"/>
       <x:c r="F170" s="62"/>
       <x:c r="G170" s="72" t="str">
-        <x:v>620BD07248317FAC18F466B0FB3C9470FF4DF1285FBE9AD0A4A3A139A5D3F3361</x:v>
+        <x:v>620BD07248317FAC18F466B0FB3C9470FF4DF1285FBE9AD0A4A3A139A5D3F361</x:v>
       </x:c>
       <x:c r="H170" s="62" t="str">
         <x:v>事务证据</x:v>
       </x:c>
       <x:c r="I170" s="70" t="n">
-        <x:v>46256</x:v>
+        <x:v>46267</x:v>
       </x:c>
       <x:c r="J170" s="63" t="str">
-        <x:v>65/65真实WZL导出回读通过</x:v>
+        <x:v>依事务原件纠正旧文档多转录的1个3；本值为64位SHA256</x:v>
       </x:c>
     </x:row>
     <x:row r="171">
@@ -11394,6 +12253,1506 @@
       </x:c>
       <x:c r="J176" t="str">
         <x:v>完整成果目录原包</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="177" ht="30" customHeight="1">
+      <x:c r="A177" s="82" t="str">
+        <x:v>EL-PARAM-FATE-SLOTS</x:v>
+      </x:c>
+      <x:c r="B177" s="83" t="str">
+        <x:v>命格</x:v>
+      </x:c>
+      <x:c r="C177" s="83" t="str">
+        <x:v>最大槽位数</x:v>
+      </x:c>
+      <x:c r="D177" s="83" t="str">
+        <x:v>槽</x:v>
+      </x:c>
+      <x:c r="E177" s="83" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F177" s="83" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G177" s="83" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H177" s="91" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="I177" s="94" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="J177" s="84" t="str">
+        <x:v>逐槽独立洗练</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="178" ht="30" customHeight="1">
+      <x:c r="A178" s="85" t="str">
+        <x:v>EL-PARAM-FATE-TIER-COUNT</x:v>
+      </x:c>
+      <x:c r="B178" s="86" t="str">
+        <x:v>命格</x:v>
+      </x:c>
+      <x:c r="C178" s="86" t="str">
+        <x:v>每档命格数量</x:v>
+      </x:c>
+      <x:c r="D178" s="86" t="str">
+        <x:v>个</x:v>
+      </x:c>
+      <x:c r="E178" s="86" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F178" s="86" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G178" s="86" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="H178" s="92" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="I178" s="95" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="J178" s="87" t="str">
+        <x:v>绿黄橙红彩各20</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="179" ht="30" customHeight="1">
+      <x:c r="A179" s="85" t="str">
+        <x:v>EL-PARAM-FATE-TOTAL</x:v>
+      </x:c>
+      <x:c r="B179" s="86" t="str">
+        <x:v>命格</x:v>
+      </x:c>
+      <x:c r="C179" s="86" t="str">
+        <x:v>五档命格总数</x:v>
+      </x:c>
+      <x:c r="D179" s="86" t="str">
+        <x:v>个</x:v>
+      </x:c>
+      <x:c r="E179" s="86" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="F179" s="86" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="G179" s="86" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="H179" s="92" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="I179" s="95" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="J179" s="87" t="str">
+        <x:v>现行权威表</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="180" ht="30" customHeight="1">
+      <x:c r="A180" s="85" t="str">
+        <x:v>EL-PARAM-FATE-STRENGTH-G</x:v>
+      </x:c>
+      <x:c r="B180" s="86" t="str">
+        <x:v>命格</x:v>
+      </x:c>
+      <x:c r="C180" s="86" t="str">
+        <x:v>绿色强度基准</x:v>
+      </x:c>
+      <x:c r="D180" s="86" t="str">
+        <x:v>级</x:v>
+      </x:c>
+      <x:c r="E180" s="86" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F180" s="86" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G180" s="86" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H180" s="92" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="I180" s="95" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="J180" s="87" t="str">
+        <x:v>相对强度</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="181" ht="30" customHeight="1">
+      <x:c r="A181" s="85" t="str">
+        <x:v>EL-PARAM-FATE-STRENGTH-Y</x:v>
+      </x:c>
+      <x:c r="B181" s="86" t="str">
+        <x:v>命格</x:v>
+      </x:c>
+      <x:c r="C181" s="86" t="str">
+        <x:v>黄色强度基准</x:v>
+      </x:c>
+      <x:c r="D181" s="86" t="str">
+        <x:v>级</x:v>
+      </x:c>
+      <x:c r="E181" s="86" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F181" s="86" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G181" s="86" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H181" s="92" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="I181" s="95" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="J181" s="87" t="str">
+        <x:v>相对强度</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="182" ht="30" customHeight="1">
+      <x:c r="A182" s="85" t="str">
+        <x:v>EL-PARAM-FATE-STRENGTH-O</x:v>
+      </x:c>
+      <x:c r="B182" s="86" t="str">
+        <x:v>命格</x:v>
+      </x:c>
+      <x:c r="C182" s="86" t="str">
+        <x:v>橙色强度基准</x:v>
+      </x:c>
+      <x:c r="D182" s="86" t="str">
+        <x:v>级</x:v>
+      </x:c>
+      <x:c r="E182" s="86" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F182" s="86" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G182" s="86" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H182" s="92" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="I182" s="95" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="J182" s="87" t="str">
+        <x:v>橙色起允许稀有词条</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="183" ht="30" customHeight="1">
+      <x:c r="A183" s="85" t="str">
+        <x:v>EL-PARAM-FATE-STRENGTH-R</x:v>
+      </x:c>
+      <x:c r="B183" s="86" t="str">
+        <x:v>命格</x:v>
+      </x:c>
+      <x:c r="C183" s="86" t="str">
+        <x:v>红色强度基准</x:v>
+      </x:c>
+      <x:c r="D183" s="86" t="str">
+        <x:v>级</x:v>
+      </x:c>
+      <x:c r="E183" s="86" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F183" s="86" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G183" s="86" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H183" s="92" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="I183" s="95" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="J183" s="87" t="str">
+        <x:v>相对强度</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="184" ht="30" customHeight="1">
+      <x:c r="A184" s="85" t="str">
+        <x:v>EL-PARAM-FATE-STRENGTH-C</x:v>
+      </x:c>
+      <x:c r="B184" s="86" t="str">
+        <x:v>命格</x:v>
+      </x:c>
+      <x:c r="C184" s="86" t="str">
+        <x:v>彩色强度基准</x:v>
+      </x:c>
+      <x:c r="D184" s="86" t="str">
+        <x:v>级</x:v>
+      </x:c>
+      <x:c r="E184" s="86" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F184" s="86" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="G184" s="86" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H184" s="92" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="I184" s="95" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="J184" s="87" t="str">
+        <x:v>明显优于红色</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="185" ht="30" customHeight="1">
+      <x:c r="A185" s="85" t="str">
+        <x:v>EL-PARAM-FATE-PITY-RED</x:v>
+      </x:c>
+      <x:c r="B185" s="86" t="str">
+        <x:v>命格</x:v>
+      </x:c>
+      <x:c r="C185" s="86" t="str">
+        <x:v>必出红色次数</x:v>
+      </x:c>
+      <x:c r="D185" s="86" t="str">
+        <x:v>次/槽</x:v>
+      </x:c>
+      <x:c r="E185" s="86" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F185" s="86" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G185" s="86" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="H185" s="92" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="I185" s="95" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="J185" s="87" t="str">
+        <x:v>独立保底</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="186" ht="30" customHeight="1">
+      <x:c r="A186" s="85" t="str">
+        <x:v>EL-PARAM-FATE-COLOR-CHECK</x:v>
+      </x:c>
+      <x:c r="B186" s="86" t="str">
+        <x:v>命格</x:v>
+      </x:c>
+      <x:c r="C186" s="86" t="str">
+        <x:v>彩色判定间隔</x:v>
+      </x:c>
+      <x:c r="D186" s="86" t="str">
+        <x:v>次/槽</x:v>
+      </x:c>
+      <x:c r="E186" s="86" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F186" s="86" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G186" s="86" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H186" s="92" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="I186" s="95" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="J186" s="87" t="str">
+        <x:v>每10次参与彩色判定</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="187" ht="30" customHeight="1">
+      <x:c r="A187" s="85" t="str">
+        <x:v>EL-PARAM-FATE-PITY-COLOR</x:v>
+      </x:c>
+      <x:c r="B187" s="86" t="str">
+        <x:v>命格</x:v>
+      </x:c>
+      <x:c r="C187" s="86" t="str">
+        <x:v>必出彩色次数</x:v>
+      </x:c>
+      <x:c r="D187" s="86" t="str">
+        <x:v>次/槽</x:v>
+      </x:c>
+      <x:c r="E187" s="86" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="F187" s="86" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="G187" s="86" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="H187" s="92" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="I187" s="95" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="J187" s="87" t="str">
+        <x:v>独立保底</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="188" ht="30" customHeight="1">
+      <x:c r="A188" s="85" t="str">
+        <x:v>EL-PARAM-FATE-COLOR-RARE</x:v>
+      </x:c>
+      <x:c r="B188" s="86" t="str">
+        <x:v>命格</x:v>
+      </x:c>
+      <x:c r="C188" s="86" t="str">
+        <x:v>彩色最大稀有词条</x:v>
+      </x:c>
+      <x:c r="D188" s="86" t="str">
+        <x:v>条</x:v>
+      </x:c>
+      <x:c r="E188" s="86" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F188" s="86" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G188" s="86" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H188" s="92" t="str">
+        <x:v>上限已确认</x:v>
+      </x:c>
+      <x:c r="I188" s="95" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="J188" s="87" t="str">
+        <x:v>具体条数按实战强度</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="189" ht="30" customHeight="1">
+      <x:c r="A189" s="85" t="str">
+        <x:v>EL-PARAM-ATKSPEED-NORMAL-CAP</x:v>
+      </x:c>
+      <x:c r="B189" s="86" t="str">
+        <x:v>攻速突破</x:v>
+      </x:c>
+      <x:c r="C189" s="86" t="str">
+        <x:v>普通攻速上限</x:v>
+      </x:c>
+      <x:c r="D189" s="86" t="str">
+        <x:v>点</x:v>
+      </x:c>
+      <x:c r="E189" s="86" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F189" s="86" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G189" s="86" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="H189" s="92" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="I189" s="95" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="J189" s="87" t="str">
+        <x:v>无突破时的端上限</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="190" ht="30" customHeight="1">
+      <x:c r="A190" s="85" t="str">
+        <x:v>EL-PARAM-ATKSPEED-BREAK-CAP</x:v>
+      </x:c>
+      <x:c r="B190" s="86" t="str">
+        <x:v>攻速突破</x:v>
+      </x:c>
+      <x:c r="C190" s="86" t="str">
+        <x:v>攻速突破技术上限</x:v>
+      </x:c>
+      <x:c r="D190" s="86" t="str">
+        <x:v>点</x:v>
+      </x:c>
+      <x:c r="E190" s="86" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="F190" s="86" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="G190" s="86" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="H190" s="92" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="I190" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="J190" s="87" t="str">
+        <x:v>技术上限30；现版本内容合计约投放20点</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="191" ht="30" customHeight="1">
+      <x:c r="A191" s="85" t="str">
+        <x:v>EL-PARAM-ATKSPEED-ACTUAL-CAP</x:v>
+      </x:c>
+      <x:c r="B191" s="86" t="str">
+        <x:v>攻速突破</x:v>
+      </x:c>
+      <x:c r="C191" s="86" t="str">
+        <x:v>生效攻速点理论上限</x:v>
+      </x:c>
+      <x:c r="D191" s="86" t="str">
+        <x:v>点</x:v>
+      </x:c>
+      <x:c r="E191" s="86" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F191" s="86" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="G191" s="86" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="H191" s="92" t="str">
+        <x:v>技术上限已确认</x:v>
+      </x:c>
+      <x:c r="I191" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="J191" s="87" t="str">
+        <x:v>20普通＋30突破；不表示现版本实际可获得50点</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="192" ht="30" customHeight="1">
+      <x:c r="A192" s="85" t="str">
+        <x:v>EL-PARAM-AOE-ZODIAC-LV1-SIZE</x:v>
+      </x:c>
+      <x:c r="B192" s="86" t="str">
+        <x:v>群攻生肖</x:v>
+      </x:c>
+      <x:c r="C192" s="86" t="str">
+        <x:v>LV1范围边长</x:v>
+      </x:c>
+      <x:c r="D192" s="86" t="str">
+        <x:v>格</x:v>
+      </x:c>
+      <x:c r="E192" s="86" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F192" s="86" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G192" s="86" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H192" s="92" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="I192" s="95" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="J192" s="87" t="str">
+        <x:v>2×2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="193" ht="30" customHeight="1">
+      <x:c r="A193" s="85" t="str">
+        <x:v>EL-PARAM-AOE-ZODIAC-LV1-CD</x:v>
+      </x:c>
+      <x:c r="B193" s="86" t="str">
+        <x:v>群攻生肖</x:v>
+      </x:c>
+      <x:c r="C193" s="86" t="str">
+        <x:v>LV1伤害间隔</x:v>
+      </x:c>
+      <x:c r="D193" s="86" t="str">
+        <x:v>秒</x:v>
+      </x:c>
+      <x:c r="E193" s="86" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F193" s="86" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G193" s="86" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H193" s="92" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="I193" s="95" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="J193" s="87" t="str">
+        <x:v>伤害为自身攻击力</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="194" ht="30" customHeight="1">
+      <x:c r="A194" s="85" t="str">
+        <x:v>EL-PARAM-AOE-ZODIAC-LV5-SIZE</x:v>
+      </x:c>
+      <x:c r="B194" s="86" t="str">
+        <x:v>群攻生肖</x:v>
+      </x:c>
+      <x:c r="C194" s="86" t="str">
+        <x:v>LV5范围边长</x:v>
+      </x:c>
+      <x:c r="D194" s="86" t="str">
+        <x:v>格</x:v>
+      </x:c>
+      <x:c r="E194" s="86" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F194" s="86" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G194" s="86" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H194" s="92" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="I194" s="95" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="J194" s="87" t="str">
+        <x:v>3×3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="195" ht="30" customHeight="1">
+      <x:c r="A195" s="85" t="str">
+        <x:v>EL-PARAM-AOE-ZODIAC-LV5-CD</x:v>
+      </x:c>
+      <x:c r="B195" s="86" t="str">
+        <x:v>群攻生肖</x:v>
+      </x:c>
+      <x:c r="C195" s="86" t="str">
+        <x:v>LV5伤害间隔</x:v>
+      </x:c>
+      <x:c r="D195" s="86" t="str">
+        <x:v>秒</x:v>
+      </x:c>
+      <x:c r="E195" s="86" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F195" s="86" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G195" s="86" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H195" s="92" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="I195" s="95" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="J195" s="87" t="str">
+        <x:v>最终档</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="196" ht="30" customHeight="1">
+      <x:c r="A196" s="85" t="str">
+        <x:v>EL-PARAM-REBIRTH-TOTAL</x:v>
+      </x:c>
+      <x:c r="B196" s="86" t="str">
+        <x:v>转生</x:v>
+      </x:c>
+      <x:c r="C196" s="86" t="str">
+        <x:v>现行转生总等级</x:v>
+      </x:c>
+      <x:c r="D196" s="86" t="str">
+        <x:v>转</x:v>
+      </x:c>
+      <x:c r="E196" s="86" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F196" s="86" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G196" s="86" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="H196" s="92" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="I196" s="95" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="J196" s="87" t="str">
+        <x:v>第4／6／8／10大陆</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="197" ht="30" customHeight="1">
+      <x:c r="A197" s="85" t="str">
+        <x:v>EL-PARAM-REBIRTH-PER-NPC</x:v>
+      </x:c>
+      <x:c r="B197" s="86" t="str">
+        <x:v>转生</x:v>
+      </x:c>
+      <x:c r="C197" s="86" t="str">
+        <x:v>每名转生NPC负责等级</x:v>
+      </x:c>
+      <x:c r="D197" s="86" t="str">
+        <x:v>转</x:v>
+      </x:c>
+      <x:c r="E197" s="86" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F197" s="86" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G197" s="86" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H197" s="92" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="I197" s="95" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="J197" s="87" t="str">
+        <x:v>共4名NPC</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="198" ht="30" customHeight="1">
+      <x:c r="A198" s="85" t="str">
+        <x:v>EL-PARAM-COLLECT-CONSUME</x:v>
+      </x:c>
+      <x:c r="B198" s="86" t="str">
+        <x:v>图鉴</x:v>
+      </x:c>
+      <x:c r="C198" s="86" t="str">
+        <x:v>每次登记消耗实物</x:v>
+      </x:c>
+      <x:c r="D198" s="86" t="str">
+        <x:v>件</x:v>
+      </x:c>
+      <x:c r="E198" s="86" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F198" s="86" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G198" s="86" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H198" s="92" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="I198" s="95" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="J198" s="87" t="str">
+        <x:v>专属装备与大陆专属材料均适用</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="199" ht="30" customHeight="1">
+      <x:c r="A199" s="88" t="str">
+        <x:v>EL-PARAM-COLLECT-CURRENCY</x:v>
+      </x:c>
+      <x:c r="B199" s="89" t="str">
+        <x:v>图鉴</x:v>
+      </x:c>
+      <x:c r="C199" s="89" t="str">
+        <x:v>登记货币消耗</x:v>
+      </x:c>
+      <x:c r="D199" s="89" t="str">
+        <x:v>金币／元宝／灵符</x:v>
+      </x:c>
+      <x:c r="E199" s="89" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F199" s="89" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G199" s="89" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H199" s="93" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="I199" s="96" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="J199" s="90" t="str">
+        <x:v>图鉴不收货币</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="200" ht="34" customHeight="1">
+      <x:c r="A200" s="82" t="str">
+        <x:v>EL-PARAM-ATKSPEED-S0-HPS</x:v>
+      </x:c>
+      <x:c r="B200" s="83" t="str">
+        <x:v>攻速实测</x:v>
+      </x:c>
+      <x:c r="C200" s="83" t="str">
+        <x:v>S_eff=0实测刀速</x:v>
+      </x:c>
+      <x:c r="D200" s="83" t="str">
+        <x:v>刀/秒</x:v>
+      </x:c>
+      <x:c r="E200" s="103" t="n">
+        <x:v>1.75</x:v>
+      </x:c>
+      <x:c r="F200" s="103" t="n">
+        <x:v>1.75</x:v>
+      </x:c>
+      <x:c r="G200" s="103" t="n">
+        <x:v>1.75</x:v>
+      </x:c>
+      <x:c r="H200" s="100" t="str">
+        <x:v>已实测</x:v>
+      </x:c>
+      <x:c r="I200" s="94" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="J200" s="84" t="str">
+        <x:v>571.429ms；10秒17/18刀两轮平均</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="201" ht="34" customHeight="1">
+      <x:c r="A201" s="85" t="str">
+        <x:v>EL-PARAM-ATKSPEED-S10-HPS</x:v>
+      </x:c>
+      <x:c r="B201" s="86" t="str">
+        <x:v>攻速实测</x:v>
+      </x:c>
+      <x:c r="C201" s="86" t="str">
+        <x:v>S_eff=10实测刀速</x:v>
+      </x:c>
+      <x:c r="D201" s="86" t="str">
+        <x:v>刀/秒</x:v>
+      </x:c>
+      <x:c r="E201" s="104" t="n">
+        <x:v>2.2</x:v>
+      </x:c>
+      <x:c r="F201" s="104" t="n">
+        <x:v>2.2</x:v>
+      </x:c>
+      <x:c r="G201" s="104" t="n">
+        <x:v>2.2</x:v>
+      </x:c>
+      <x:c r="H201" s="101" t="str">
+        <x:v>已实测</x:v>
+      </x:c>
+      <x:c r="I201" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="J201" s="87" t="str">
+        <x:v>454.545ms；10秒22刀</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="202" ht="34" customHeight="1">
+      <x:c r="A202" s="85" t="str">
+        <x:v>EL-PARAM-ATKSPEED-S20-HPS</x:v>
+      </x:c>
+      <x:c r="B202" s="86" t="str">
+        <x:v>攻速实测</x:v>
+      </x:c>
+      <x:c r="C202" s="86" t="str">
+        <x:v>S_eff=20实测刀速</x:v>
+      </x:c>
+      <x:c r="D202" s="86" t="str">
+        <x:v>刀/秒</x:v>
+      </x:c>
+      <x:c r="E202" s="104" t="n">
+        <x:v>2.9</x:v>
+      </x:c>
+      <x:c r="F202" s="104" t="n">
+        <x:v>2.9</x:v>
+      </x:c>
+      <x:c r="G202" s="104" t="n">
+        <x:v>2.9</x:v>
+      </x:c>
+      <x:c r="H202" s="101" t="str">
+        <x:v>已实测</x:v>
+      </x:c>
+      <x:c r="I202" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="J202" s="87" t="str">
+        <x:v>344.828ms；10秒29刀</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="203" ht="34" customHeight="1">
+      <x:c r="A203" s="85" t="str">
+        <x:v>EL-PARAM-ATKSPEED-S30-HPS</x:v>
+      </x:c>
+      <x:c r="B203" s="86" t="str">
+        <x:v>攻速实测</x:v>
+      </x:c>
+      <x:c r="C203" s="86" t="str">
+        <x:v>S_eff=30实测刀速</x:v>
+      </x:c>
+      <x:c r="D203" s="86" t="str">
+        <x:v>刀/秒</x:v>
+      </x:c>
+      <x:c r="E203" s="104" t="n">
+        <x:v>4.3</x:v>
+      </x:c>
+      <x:c r="F203" s="104" t="n">
+        <x:v>4.3</x:v>
+      </x:c>
+      <x:c r="G203" s="104" t="n">
+        <x:v>4.3</x:v>
+      </x:c>
+      <x:c r="H203" s="101" t="str">
+        <x:v>已实测</x:v>
+      </x:c>
+      <x:c r="I203" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="J203" s="87" t="str">
+        <x:v>232.558ms；10秒43刀</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="204" ht="34" customHeight="1">
+      <x:c r="A204" s="85" t="str">
+        <x:v>EL-PARAM-ATKSPEED-S40-HPS</x:v>
+      </x:c>
+      <x:c r="B204" s="86" t="str">
+        <x:v>攻速实测</x:v>
+      </x:c>
+      <x:c r="C204" s="86" t="str">
+        <x:v>S_eff=40实测刀速</x:v>
+      </x:c>
+      <x:c r="D204" s="86" t="str">
+        <x:v>刀/秒</x:v>
+      </x:c>
+      <x:c r="E204" s="104" t="n">
+        <x:v>8.5</x:v>
+      </x:c>
+      <x:c r="F204" s="104" t="n">
+        <x:v>8.5</x:v>
+      </x:c>
+      <x:c r="G204" s="104" t="n">
+        <x:v>8.5</x:v>
+      </x:c>
+      <x:c r="H204" s="101" t="str">
+        <x:v>已实测</x:v>
+      </x:c>
+      <x:c r="I204" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="J204" s="87" t="str">
+        <x:v>117.647ms；10秒85刀</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="205" ht="34" customHeight="1">
+      <x:c r="A205" s="85" t="str">
+        <x:v>EL-PARAM-ATKSPEED-S50-HPS</x:v>
+      </x:c>
+      <x:c r="B205" s="86" t="str">
+        <x:v>攻速实测</x:v>
+      </x:c>
+      <x:c r="C205" s="86" t="str">
+        <x:v>S_eff=50实测刀速</x:v>
+      </x:c>
+      <x:c r="D205" s="86" t="str">
+        <x:v>刀/秒</x:v>
+      </x:c>
+      <x:c r="E205" s="104" t="n">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="F205" s="104" t="n">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="G205" s="104" t="n">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="H205" s="101" t="str">
+        <x:v>已实测（单点）</x:v>
+      </x:c>
+      <x:c r="I205" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="J205" s="87" t="str">
+        <x:v>69.930ms；10秒143刀；不证明引擎天然硬上限</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="206" ht="34" customHeight="1">
+      <x:c r="A206" s="85" t="str">
+        <x:v>EL-PARAM-ATKSPEED-FIT-A</x:v>
+      </x:c>
+      <x:c r="B206" s="86" t="str">
+        <x:v>攻速公式</x:v>
+      </x:c>
+      <x:c r="C206" s="86" t="str">
+        <x:v>0—40档刀间隔截距</x:v>
+      </x:c>
+      <x:c r="D206" s="86" t="str">
+        <x:v>ms</x:v>
+      </x:c>
+      <x:c r="E206" s="104" t="n">
+        <x:v>570.11143</x:v>
+      </x:c>
+      <x:c r="F206" s="104" t="n">
+        <x:v>570.11143</x:v>
+      </x:c>
+      <x:c r="G206" s="104" t="n">
+        <x:v>570.11143</x:v>
+      </x:c>
+      <x:c r="H206" s="101" t="str">
+        <x:v>已实测拟合</x:v>
+      </x:c>
+      <x:c r="I206" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="J206" s="87" t="str">
+        <x:v>T=570.111430-11.295503×S_eff</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="207" ht="34" customHeight="1">
+      <x:c r="A207" s="85" t="str">
+        <x:v>EL-PARAM-ATKSPEED-FIT-B</x:v>
+      </x:c>
+      <x:c r="B207" s="86" t="str">
+        <x:v>攻速公式</x:v>
+      </x:c>
+      <x:c r="C207" s="86" t="str">
+        <x:v>0—40档每点间隔减少</x:v>
+      </x:c>
+      <x:c r="D207" s="86" t="str">
+        <x:v>ms/点</x:v>
+      </x:c>
+      <x:c r="E207" s="104" t="n">
+        <x:v>11.295503</x:v>
+      </x:c>
+      <x:c r="F207" s="104" t="n">
+        <x:v>11.295503</x:v>
+      </x:c>
+      <x:c r="G207" s="104" t="n">
+        <x:v>11.295503</x:v>
+      </x:c>
+      <x:c r="H207" s="101" t="str">
+        <x:v>已实测拟合</x:v>
+      </x:c>
+      <x:c r="I207" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="J207" s="87" t="str">
+        <x:v>公式中以减法使用</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="208" ht="34" customHeight="1">
+      <x:c r="A208" s="85" t="str">
+        <x:v>EL-PARAM-ATKSPEED-FIT-R2</x:v>
+      </x:c>
+      <x:c r="B208" s="86" t="str">
+        <x:v>攻速公式</x:v>
+      </x:c>
+      <x:c r="C208" s="86" t="str">
+        <x:v>0—40档拟合R²</x:v>
+      </x:c>
+      <x:c r="D208" s="86" t="str">
+        <x:v>比例</x:v>
+      </x:c>
+      <x:c r="E208" s="104" t="n">
+        <x:v>0.99991317</x:v>
+      </x:c>
+      <x:c r="F208" s="104" t="n">
+        <x:v>0.99991317</x:v>
+      </x:c>
+      <x:c r="G208" s="104" t="n">
+        <x:v>0.99991317</x:v>
+      </x:c>
+      <x:c r="H208" s="101" t="str">
+        <x:v>已实测拟合</x:v>
+      </x:c>
+      <x:c r="I208" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="J208" s="87" t="str">
+        <x:v>残差绝对值小于2.7ms</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="209" ht="34" customHeight="1">
+      <x:c r="A209" s="85" t="str">
+        <x:v>EL-PARAM-ATKSPEED-BREAK-BUDGET</x:v>
+      </x:c>
+      <x:c r="B209" s="86" t="str">
+        <x:v>攻速突破</x:v>
+      </x:c>
+      <x:c r="C209" s="86" t="str">
+        <x:v>现版本全程突破投放总量</x:v>
+      </x:c>
+      <x:c r="D209" s="86" t="str">
+        <x:v>点</x:v>
+      </x:c>
+      <x:c r="E209" s="86" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F209" s="86" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G209" s="86" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="H209" s="101" t="str">
+        <x:v>规划目标</x:v>
+      </x:c>
+      <x:c r="I209" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="J209" s="87" t="str">
+        <x:v>约20点；技术上限30不是投放量</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="210" ht="34" customHeight="1">
+      <x:c r="A210" s="85" t="str">
+        <x:v>EL-PARAM-ATKSPEED-BREAK-FATE</x:v>
+      </x:c>
+      <x:c r="B210" s="86" t="str">
+        <x:v>攻速突破</x:v>
+      </x:c>
+      <x:c r="C210" s="86" t="str">
+        <x:v>命格渠道投放</x:v>
+      </x:c>
+      <x:c r="D210" s="86" t="str">
+        <x:v>点</x:v>
+      </x:c>
+      <x:c r="E210" s="86" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F210" s="86" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G210" s="86" t="str">
+        <x:v>3—5</x:v>
+      </x:c>
+      <x:c r="H210" s="101" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="I210" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="J210" s="87" t="str">
+        <x:v>指命格渠道合计预算，不自动解读为每条命格</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="211" ht="34" customHeight="1">
+      <x:c r="A211" s="85" t="str">
+        <x:v>EL-PARAM-ATKSPEED-BREAK-WEAPON</x:v>
+      </x:c>
+      <x:c r="B211" s="86" t="str">
+        <x:v>攻速突破</x:v>
+      </x:c>
+      <x:c r="C211" s="86" t="str">
+        <x:v>单把武器突破上限</x:v>
+      </x:c>
+      <x:c r="D211" s="86" t="str">
+        <x:v>点</x:v>
+      </x:c>
+      <x:c r="E211" s="86" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F211" s="86" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G211" s="86" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H211" s="101" t="str">
+        <x:v>上限已确认</x:v>
+      </x:c>
+      <x:c r="I211" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="J211" s="87" t="str">
+        <x:v>按武器稀有度投放；非所有武器都给5点</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="212" ht="34" customHeight="1">
+      <x:c r="A212" s="88" t="str">
+        <x:v>EL-PARAM-CRIT-BASE-MULT</x:v>
+      </x:c>
+      <x:c r="B212" s="89" t="str">
+        <x:v>暴击期望</x:v>
+      </x:c>
+      <x:c r="C212" s="89" t="str">
+        <x:v>基础暴击总倍率</x:v>
+      </x:c>
+      <x:c r="D212" s="89" t="str">
+        <x:v>倍</x:v>
+      </x:c>
+      <x:c r="E212" s="89"/>
+      <x:c r="F212" s="89"/>
+      <x:c r="G212" s="89" t="str">
+        <x:v>待引擎确认</x:v>
+      </x:c>
+      <x:c r="H212" s="102" t="str">
+        <x:v>待确认</x:v>
+      </x:c>
+      <x:c r="I212" s="96" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="J212" s="90" t="str">
+        <x:v>旧参考档记载2倍，现行不直接当正式值</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="213" ht="32" customHeight="1">
+      <x:c r="A213" s="82" t="str">
+        <x:v>EL-PARAM-C3C10-CONTINENTS</x:v>
+      </x:c>
+      <x:c r="B213" s="83" t="str">
+        <x:v>内容结构</x:v>
+      </x:c>
+      <x:c r="C213" s="83" t="str">
+        <x:v>第3—10大陆数量</x:v>
+      </x:c>
+      <x:c r="D213" s="83" t="str">
+        <x:v>个</x:v>
+      </x:c>
+      <x:c r="E213" s="83" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F213" s="83" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G213" s="83" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H213" s="105" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="I213" s="94" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="J213" s="84" t="str">
+        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.0.xlsx</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="214" ht="32" customHeight="1">
+      <x:c r="A214" s="85" t="str">
+        <x:v>EL-PARAM-C3C10-GROUPS</x:v>
+      </x:c>
+      <x:c r="B214" s="86" t="str">
+        <x:v>内容结构</x:v>
+      </x:c>
+      <x:c r="C214" s="86" t="str">
+        <x:v>第3—10大陆地图组</x:v>
+      </x:c>
+      <x:c r="D214" s="86" t="str">
+        <x:v>组</x:v>
+      </x:c>
+      <x:c r="E214" s="86" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="F214" s="86" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="G214" s="86" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="H214" s="106" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="I214" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="J214" s="87" t="str">
+        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.0.xlsx</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="215" ht="32" customHeight="1">
+      <x:c r="A215" s="85" t="str">
+        <x:v>EL-PARAM-C3C10-MAPS</x:v>
+      </x:c>
+      <x:c r="B215" s="86" t="str">
+        <x:v>内容结构</x:v>
+      </x:c>
+      <x:c r="C215" s="86" t="str">
+        <x:v>第3—10大陆地图</x:v>
+      </x:c>
+      <x:c r="D215" s="86" t="str">
+        <x:v>张</x:v>
+      </x:c>
+      <x:c r="E215" s="86" t="n">
+        <x:v>144</x:v>
+      </x:c>
+      <x:c r="F215" s="86" t="n">
+        <x:v>144</x:v>
+      </x:c>
+      <x:c r="G215" s="86" t="n">
+        <x:v>144</x:v>
+      </x:c>
+      <x:c r="H215" s="106" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="I215" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="J215" s="87" t="str">
+        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.0.xlsx</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="216" ht="32" customHeight="1">
+      <x:c r="A216" s="85" t="str">
+        <x:v>EL-PARAM-C3C10-MONSTERS</x:v>
+      </x:c>
+      <x:c r="B216" s="86" t="str">
+        <x:v>内容结构</x:v>
+      </x:c>
+      <x:c r="C216" s="86" t="str">
+        <x:v>第3—10大陆怪物总数</x:v>
+      </x:c>
+      <x:c r="D216" s="86" t="str">
+        <x:v>只</x:v>
+      </x:c>
+      <x:c r="E216" s="86" t="n">
+        <x:v>464</x:v>
+      </x:c>
+      <x:c r="F216" s="86" t="n">
+        <x:v>464</x:v>
+      </x:c>
+      <x:c r="G216" s="86" t="n">
+        <x:v>464</x:v>
+      </x:c>
+      <x:c r="H216" s="106" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="I216" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="J216" s="87" t="str">
+        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.0.xlsx</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="217" ht="32" customHeight="1">
+      <x:c r="A217" s="85" t="str">
+        <x:v>EL-PARAM-C3C10-NORMAL</x:v>
+      </x:c>
+      <x:c r="B217" s="86" t="str">
+        <x:v>内容结构</x:v>
+      </x:c>
+      <x:c r="C217" s="86" t="str">
+        <x:v>普通怪</x:v>
+      </x:c>
+      <x:c r="D217" s="86" t="str">
+        <x:v>只</x:v>
+      </x:c>
+      <x:c r="E217" s="86" t="n">
+        <x:v>228</x:v>
+      </x:c>
+      <x:c r="F217" s="86" t="n">
+        <x:v>228</x:v>
+      </x:c>
+      <x:c r="G217" s="86" t="n">
+        <x:v>228</x:v>
+      </x:c>
+      <x:c r="H217" s="106" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="I217" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="J217" s="87" t="str">
+        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.0.xlsx</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="218" ht="32" customHeight="1">
+      <x:c r="A218" s="85" t="str">
+        <x:v>EL-PARAM-C3C10-RARE</x:v>
+      </x:c>
+      <x:c r="B218" s="86" t="str">
+        <x:v>内容结构</x:v>
+      </x:c>
+      <x:c r="C218" s="86" t="str">
+        <x:v>稀有怪</x:v>
+      </x:c>
+      <x:c r="D218" s="86" t="str">
+        <x:v>只</x:v>
+      </x:c>
+      <x:c r="E218" s="86" t="n">
+        <x:v>152</x:v>
+      </x:c>
+      <x:c r="F218" s="86" t="n">
+        <x:v>152</x:v>
+      </x:c>
+      <x:c r="G218" s="86" t="n">
+        <x:v>152</x:v>
+      </x:c>
+      <x:c r="H218" s="106" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="I218" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="J218" s="87" t="str">
+        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.0.xlsx</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="219" ht="32" customHeight="1">
+      <x:c r="A219" s="85" t="str">
+        <x:v>EL-PARAM-C3C10-MAPBOSS</x:v>
+      </x:c>
+      <x:c r="B219" s="86" t="str">
+        <x:v>内容结构</x:v>
+      </x:c>
+      <x:c r="C219" s="86" t="str">
+        <x:v>地图BOSS</x:v>
+      </x:c>
+      <x:c r="D219" s="86" t="str">
+        <x:v>只</x:v>
+      </x:c>
+      <x:c r="E219" s="86" t="n">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="F219" s="86" t="n">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="G219" s="86" t="n">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="H219" s="106" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="I219" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="J219" s="87" t="str">
+        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.0.xlsx</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="220" ht="32" customHeight="1">
+      <x:c r="A220" s="85" t="str">
+        <x:v>EL-PARAM-C3C10-FINALBOSS</x:v>
+      </x:c>
+      <x:c r="B220" s="86" t="str">
+        <x:v>内容结构</x:v>
+      </x:c>
+      <x:c r="C220" s="86" t="str">
+        <x:v>大陆最终BOSS</x:v>
+      </x:c>
+      <x:c r="D220" s="86" t="str">
+        <x:v>只</x:v>
+      </x:c>
+      <x:c r="E220" s="86" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F220" s="86" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G220" s="86" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H220" s="106" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="I220" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="J220" s="87" t="str">
+        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.0.xlsx</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="221" ht="32" customHeight="1">
+      <x:c r="A221" s="85" t="str">
+        <x:v>EL-PARAM-C3C10-EXCLUSIVES</x:v>
+      </x:c>
+      <x:c r="B221" s="86" t="str">
+        <x:v>内容结构</x:v>
+      </x:c>
+      <x:c r="C221" s="86" t="str">
+        <x:v>一怪一专属</x:v>
+      </x:c>
+      <x:c r="D221" s="86" t="str">
+        <x:v>件</x:v>
+      </x:c>
+      <x:c r="E221" s="86" t="n">
+        <x:v>464</x:v>
+      </x:c>
+      <x:c r="F221" s="86" t="n">
+        <x:v>464</x:v>
+      </x:c>
+      <x:c r="G221" s="86" t="n">
+        <x:v>464</x:v>
+      </x:c>
+      <x:c r="H221" s="106" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="I221" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="J221" s="87" t="str">
+        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.0.xlsx</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="222" ht="32" customHeight="1">
+      <x:c r="A222" s="85" t="str">
+        <x:v>EL-PARAM-C3C10-MATERIALS</x:v>
+      </x:c>
+      <x:c r="B222" s="86" t="str">
+        <x:v>内容结构</x:v>
+      </x:c>
+      <x:c r="C222" s="86" t="str">
+        <x:v>沿用已入库材料</x:v>
+      </x:c>
+      <x:c r="D222" s="86" t="str">
+        <x:v>件</x:v>
+      </x:c>
+      <x:c r="E222" s="86" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="F222" s="86" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="G222" s="86" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="H222" s="106" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="I222" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="J222" s="87" t="str">
+        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.0.xlsx</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="223" ht="32" customHeight="1">
+      <x:c r="A223" s="88" t="str">
+        <x:v>EL-PARAM-C3C10-COLLECTIBLES</x:v>
+      </x:c>
+      <x:c r="B223" s="89" t="str">
+        <x:v>内容结构</x:v>
+      </x:c>
+      <x:c r="C223" s="89" t="str">
+        <x:v>大陆收藏材料</x:v>
+      </x:c>
+      <x:c r="D223" s="89" t="str">
+        <x:v>件</x:v>
+      </x:c>
+      <x:c r="E223" s="89" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F223" s="89" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G223" s="89" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H223" s="107" t="str">
+        <x:v>名称已确认</x:v>
+      </x:c>
+      <x:c r="I223" s="96" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="J223" s="90" t="str">
+        <x:v>代码、爆率、奖励待定</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -12034,6 +14393,32 @@
         <x:v>原件已核验</x:v>
       </x:c>
     </x:row>
+    <x:row r="25" ht="44" customHeight="1">
+      <x:c r="A25" s="111" t="str">
+        <x:v>EL-EQUIP-C3C10-FRAME-001</x:v>
+      </x:c>
+      <x:c r="B25" s="112" t="str">
+        <x:v>定向专属</x:v>
+      </x:c>
+      <x:c r="C25" s="112" t="str">
+        <x:v>第3—10大陆464件一怪一专属</x:v>
+      </x:c>
+      <x:c r="D25" s="112" t="str">
+        <x:v>第3—10大陆</x:v>
+      </x:c>
+      <x:c r="E25" s="112" t="str">
+        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.0.xlsx</x:v>
+      </x:c>
+      <x:c r="F25" s="114" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="G25" s="112" t="str">
+        <x:v>464怪逐一对应；来源编号与正式属性待后续施工</x:v>
+      </x:c>
+      <x:c r="H25" s="113" t="str">
+        <x:v>结构定稿／待分配编码</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
@@ -12386,6 +14771,32 @@
         <x:v>修改表已生成，待Codex测试执行</x:v>
       </x:c>
     </x:row>
+    <x:row r="14" ht="44" customHeight="1">
+      <x:c r="A14" s="111" t="str">
+        <x:v>EL-MON-C3C10-FRAME-001</x:v>
+      </x:c>
+      <x:c r="B14" s="112" t="str">
+        <x:v>第3—10大陆怪物</x:v>
+      </x:c>
+      <x:c r="C14" s="112" t="str">
+        <x:v>C3—C10</x:v>
+      </x:c>
+      <x:c r="D14" s="112" t="str">
+        <x:v>38组／144图／464怪</x:v>
+      </x:c>
+      <x:c r="E14" s="112" t="str">
+        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.0.xlsx</x:v>
+      </x:c>
+      <x:c r="F14" s="114" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="G14" s="112" t="str">
+        <x:v>228普通＋152稀有＋76地图BOSS＋8最终BOSS</x:v>
+      </x:c>
+      <x:c r="H14" s="113" t="str">
+        <x:v>结构定稿／数值待算</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
@@ -12834,6 +15245,32 @@
         <x:v>位置原则已确认</x:v>
       </x:c>
     </x:row>
+    <x:row r="18" ht="44" customHeight="1">
+      <x:c r="A18" s="111" t="str">
+        <x:v>EL-MAP-C3C10-MONSTER-FRAME-001</x:v>
+      </x:c>
+      <x:c r="B18" s="112" t="str">
+        <x:v>第3—10大陆怪物部署</x:v>
+      </x:c>
+      <x:c r="C18" s="112" t="str">
+        <x:v>C3—C10</x:v>
+      </x:c>
+      <x:c r="D18" s="112" t="str">
+        <x:v>38组／144图</x:v>
+      </x:c>
+      <x:c r="E18" s="112" t="str">
+        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.0.xlsx</x:v>
+      </x:c>
+      <x:c r="F18" s="114" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="G18" s="112" t="str">
+        <x:v>464怪全部对应准确地图；雾月水庭名称已纠正</x:v>
+      </x:c>
+      <x:c r="H18" s="113" t="str">
+        <x:v>地图冻结／分怪完成</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
@@ -13204,6 +15641,58 @@
         <x:v>原件已接续／65条逐行通过／游戏内待验收</x:v>
       </x:c>
     </x:row>
+    <x:row r="15" ht="44" customHeight="1">
+      <x:c r="A15" s="82" t="str">
+        <x:v>EL-DROP-C3C10-POOLS-001</x:v>
+      </x:c>
+      <x:c r="B15" s="83" t="str">
+        <x:v>第3—10大陆全部怪物</x:v>
+      </x:c>
+      <x:c r="C15" s="83" t="str">
+        <x:v>自身专属／BOSS兼掉／既有材料／大陆收藏／追梦神器</x:v>
+      </x:c>
+      <x:c r="D15" s="83" t="str">
+        <x:v>五类独立池</x:v>
+      </x:c>
+      <x:c r="E15" s="83" t="str">
+        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.0.xlsx</x:v>
+      </x:c>
+      <x:c r="F15" s="94" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="G15" s="83" t="str">
+        <x:v>分别配置与核算</x:v>
+      </x:c>
+      <x:c r="H15" s="84" t="str">
+        <x:v>结构定稿／概率待算</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="44" customHeight="1">
+      <x:c r="A16" s="88" t="str">
+        <x:v>EL-DROP-C3C10-MATERIALS-001</x:v>
+      </x:c>
+      <x:c r="B16" s="89" t="str">
+        <x:v>第3—10大陆全部怪物</x:v>
+      </x:c>
+      <x:c r="C16" s="89" t="str">
+        <x:v>56件既有材料＋8件大陆收藏材料</x:v>
+      </x:c>
+      <x:c r="D16" s="89" t="str">
+        <x:v>按大陆来源</x:v>
+      </x:c>
+      <x:c r="E16" s="89" t="str">
+        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.0.xlsx</x:v>
+      </x:c>
+      <x:c r="F16" s="96" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="G16" s="89" t="str">
+        <x:v>既有材料Idx 916—971；收藏材料代码待取</x:v>
+      </x:c>
+      <x:c r="H16" s="90" t="str">
+        <x:v>名称与来源定稿／概率待算</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>

</xml_diff>

<commit_message>
Allocate C3-C10 exclusive and material codes
</commit_message>
<xml_diff>
--- a/codex_tasks/艾尔登法环_第一二大陆_Codex施工包_20260821/项目档案/02_已确认规则与数值.xlsx
+++ b/codex_tasks/艾尔登法环_第一二大陆_Codex施工包_20260821/项目档案/02_已确认规则与数值.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R653ac072bb0b44a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="已确认规则" sheetId="2" r:id="Rb0a53c0427894aea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数值参数" sheetId="3" r:id="R5de56a3967c2496e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="装备索引" sheetId="4" r:id="Rb2692fbada684464"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="怪物索引" sheetId="5" r:id="R32640b05a2ae469d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="地图索引" sheetId="6" r:id="Rf2e5f13c0e4c40fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="掉落索引" sheetId="7" r:id="Ref021a6b8a244d96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R3ecdcf77fd834501"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="已确认规则" sheetId="2" r:id="R933413263fbf43b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数值参数" sheetId="3" r:id="R3c340fc60e464340"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="装备索引" sheetId="4" r:id="Rf0a15f740cbb4215"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="怪物索引" sheetId="5" r:id="Ra3fdefc777554b7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="地图索引" sheetId="6" r:id="R6c1664008c134b52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="掉落索引" sheetId="7" r:id="Ra8f648e8754742b7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -70,7 +70,7 @@
       <x:name val="Microsoft YaHei"/>
     </x:font>
   </x:fonts>
-  <x:fills count="13">
+  <x:fills count="14">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -130,6 +130,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3CD"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -274,7 +279,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="115">
+  <x:cellXfs count="118">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -558,6 +563,15 @@
     <x:xf numFmtId="200" fontId="6" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="13" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="13" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -896,7 +910,7 @@
         <x:v>当前说明</x:v>
       </x:c>
       <x:c r="B9" s="30" t="str">
-        <x:v>现行范围为10个正式大陆＋3个预留主题；功能与地图已冻结。NPC V0.2、命格100组、20转、六档攻速／TTK及第3—10大陆464怪／464专属来源框架按最新确认执行。</x:v>
+        <x:v>现行范围为10个正式大陆＋3个预留主题；怪物模型/编码由用户处理。第3—10大陆专属已阶段分配342/464码，缺122码；8件大陆收藏材料Idx 972—979已规划，Items Looks缺8个；后续成品同步GitHub。</x:v>
       </x:c>
       <x:c r="C9"/>
       <x:c r="D9"/>
@@ -5878,10 +5892,10 @@
         <x:v>材料施工</x:v>
       </x:c>
       <x:c r="C211" s="59" t="str">
-        <x:v>Idx 907—971及Items Looks 6398—6462以完整材料库原件确认为已占用，Idx 972—983为预留冻结段且占用0行。新增材料前必须查权威库并登记事务。</x:v>
+        <x:v>Idx 907—971及Items Looks 6398—6462以完整材料库原件确认为已占用。原预留Idx 972—983已于2026-09-02拆为批次B规划972—979与继续冻结980—983；新增材料前必须查权威库并登记新事务。</x:v>
       </x:c>
       <x:c r="D211" s="59" t="str">
-        <x:v>原件已确认／占用与预留冻结继续生效</x:v>
+        <x:v>批次A占用确认／批次B规划生效</x:v>
       </x:c>
       <x:c r="E211" s="69" t="n">
         <x:v>46256</x:v>
@@ -5890,7 +5904,7 @@
         <x:v>材料编码数据库.xlsx＋跨库核验</x:v>
       </x:c>
       <x:c r="G211" s="60" t="str">
-        <x:v>Items Looks 6398—6462与装备库同号候选存在65个确认重叠；本轮不改装备表，但暂停该段作为新装备来源编号</x:v>
+        <x:v>Items Looks 6398—6462与装备库同号候选存在65个确认重叠；批次B尚缺8个Items Looks，旧事务号不得复用</x:v>
       </x:c>
     </x:row>
     <x:row r="212" ht="44" customHeight="1">
@@ -6591,19 +6605,19 @@
         <x:v>材料来源</x:v>
       </x:c>
       <x:c r="C242" s="86" t="str">
-        <x:v>第3—10大陆沿用56件已入库材料，每大陆7件，锁定Idx 916—971、Items Looks 6407—6462；本轮只建立来源关系。</x:v>
+        <x:v>第3—10大陆沿用56件已入库材料，每大陆7件，锁定Idx 916—971、Items Looks 6407—6462；既有材料字段保持不变。</x:v>
       </x:c>
       <x:c r="D242" s="106" t="str">
-        <x:v>已确认</x:v>
+        <x:v>已确认／既有材料不变</x:v>
       </x:c>
       <x:c r="E242" s="95" t="n">
         <x:v>46267</x:v>
       </x:c>
       <x:c r="F242" s="86" t="str">
-        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.0.xlsx</x:v>
+        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.1_编码阶段分配.xlsx</x:v>
       </x:c>
       <x:c r="G242" s="87" t="str">
-        <x:v>冻结预留Idx 972—983不得直接启用</x:v>
+        <x:v>大陆收藏材料另按批次B规划Idx 972—979；Idx 980—983继续冻结</x:v>
       </x:c>
     </x:row>
     <x:row r="243" ht="46" customHeight="1">
@@ -6617,16 +6631,16 @@
         <x:v>第3—10大陆8件收藏材料名称定稿：西境风痕碑拓、月潮忆珀、湖心月谱残章、熔原罪火残章、永霜朝圣痕、穹霜碑珀、古坛鎏叶髓、穹律鎏痕拓片。</x:v>
       </x:c>
       <x:c r="D243" s="106" t="str">
-        <x:v>名称已确认</x:v>
+        <x:v>名称及Idx已规划</x:v>
       </x:c>
       <x:c r="E243" s="95" t="n">
         <x:v>46267</x:v>
       </x:c>
       <x:c r="F243" s="86" t="str">
-        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.0.xlsx</x:v>
+        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.1_编码阶段分配.xlsx</x:v>
       </x:c>
       <x:c r="G243" s="87" t="str">
-        <x:v>材料代码、基础爆率和登记奖励待资源总账</x:v>
+        <x:v>Idx 972—979已规划；Items Looks、基础爆率和登记奖励待资源总账</x:v>
       </x:c>
     </x:row>
     <x:row r="244" ht="46" customHeight="1">
@@ -6719,6 +6733,121 @@
       </x:c>
       <x:c r="G247" s="90" t="str">
         <x:v>自然掉落不足以支持全彩，全彩属于付费追求</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="248" ht="48" customHeight="1">
+      <x:c r="A248" s="82" t="str">
+        <x:v>EL-CODE-SCOPE-MONSTER-001</x:v>
+      </x:c>
+      <x:c r="B248" s="83" t="str">
+        <x:v>施工分工</x:v>
+      </x:c>
+      <x:c r="C248" s="83" t="str">
+        <x:v>怪物模型与怪物编码不由当前窗口分配；用户自行处理。当前窗口只维护怪物名称、地图关系、专属装备及材料编码。</x:v>
+      </x:c>
+      <x:c r="D248" s="115" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="E248" s="94" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="F248" s="83" t="str">
+        <x:v>2026-09-02用户最新确认</x:v>
+      </x:c>
+      <x:c r="G248" s="84" t="str">
+        <x:v>总账W列只写边界状态，不写任何怪物编码值</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="249" ht="48" customHeight="1">
+      <x:c r="A249" s="85" t="str">
+        <x:v>EL-C3C10-EXCLUSIVE-CODE-001</x:v>
+      </x:c>
+      <x:c r="B249" s="86" t="str">
+        <x:v>装备编码</x:v>
+      </x:c>
+      <x:c r="C249" s="86" t="str">
+        <x:v>第3—10大陆464件专属按部位审计后阶段分配342个来源编号；122件待补码：武器60、衣服51、斗笠11。</x:v>
+      </x:c>
+      <x:c r="D249" s="116" t="str">
+        <x:v>阶段分配完成</x:v>
+      </x:c>
+      <x:c r="E249" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="F249" s="86" t="str">
+        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.1_编码阶段分配.xlsx＋装备素材套装代码表.xlsx＋材料编码数据库.xlsx</x:v>
+      </x:c>
+      <x:c r="G249" s="87" t="str">
+        <x:v>342码内部重复0；与C1/C2现用219码交集0；与材料Looks 6398—6462交集0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="250" ht="48" customHeight="1">
+      <x:c r="A250" s="85" t="str">
+        <x:v>EL-CODE-SLOT-COMPAT-001</x:v>
+      </x:c>
+      <x:c r="B250" s="86" t="str">
+        <x:v>编码规则</x:v>
+      </x:c>
+      <x:c r="C250" s="86" t="str">
+        <x:v>装备来源编号必须按物理槽位匹配；现行模板严格按衣服→男衣服StdMode10、斗笠→面巾StdMode16/位置13。其他部位盈余不得跨槽硬凑，女衣服码未经平台确认不并入通用衣服池。</x:v>
+      </x:c>
+      <x:c r="D250" s="116" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="E250" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="F250" s="86" t="str">
+        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.1_编码阶段分配.xlsx＋装备素材套装代码表.xlsx＋材料编码数据库.xlsx</x:v>
+      </x:c>
+      <x:c r="G250" s="87" t="str">
+        <x:v>旧九部位码只作规划锁定，正式入库前仍需实库回读</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="251" ht="48" customHeight="1">
+      <x:c r="A251" s="85" t="str">
+        <x:v>EL-C3C10-MATERIAL-CODE-001</x:v>
+      </x:c>
+      <x:c r="B251" s="86" t="str">
+        <x:v>材料编码</x:v>
+      </x:c>
+      <x:c r="C251" s="86" t="str">
+        <x:v>8件大陆收藏材料启用原预留Idx 972—979作批次B规划；Items Looks仍缺8个，未写StdItems、未写Items图库、未生成事务号。Idx 980—983继续冻结。</x:v>
+      </x:c>
+      <x:c r="D251" s="116" t="str">
+        <x:v>Idx已规划／Looks待补</x:v>
+      </x:c>
+      <x:c r="E251" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="F251" s="86" t="str">
+        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.1_编码阶段分配.xlsx＋装备素材套装代码表.xlsx＋材料编码数据库.xlsx</x:v>
+      </x:c>
+      <x:c r="G251" s="87" t="str">
+        <x:v>6463—6470与装备来源候选重叠，不得机械顺延作为材料Looks</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="252" ht="48" customHeight="1">
+      <x:c r="A252" s="88" t="str">
+        <x:v>EL-GITHUB-SYNC-001</x:v>
+      </x:c>
+      <x:c r="B252" s="89" t="str">
+        <x:v>归档制度</x:v>
+      </x:c>
+      <x:c r="C252" s="89" t="str">
+        <x:v>此后当前窗口制作的正式表格、专题档案、确认记录与核心档案更新均同步到GitHub对应项目文件夹；聊天记忆不作为唯一保存介质。</x:v>
+      </x:c>
+      <x:c r="D252" s="117" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="E252" s="96" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="F252" s="89" t="str">
+        <x:v>2026-09-02用户最新确认</x:v>
+      </x:c>
+      <x:c r="G252" s="90" t="str">
+        <x:v>提交后必须回读文件清单和哈希；未提交不得声称已同步</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -13746,13 +13875,269 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="H223" s="107" t="str">
-        <x:v>名称已确认</x:v>
+        <x:v>名称及Idx已规划</x:v>
       </x:c>
       <x:c r="I223" s="96" t="n">
         <x:v>46267</x:v>
       </x:c>
       <x:c r="J223" s="90" t="str">
-        <x:v>代码、爆率、奖励待定</x:v>
+        <x:v>Idx 972—979；Items Looks、爆率、奖励待定</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="224" ht="36" customHeight="1">
+      <x:c r="A224" s="82" t="str">
+        <x:v>EL-PARAM-C3C10-CODE-DEMAND</x:v>
+      </x:c>
+      <x:c r="B224" s="83" t="str">
+        <x:v>编码资源</x:v>
+      </x:c>
+      <x:c r="C224" s="83" t="str">
+        <x:v>C3—C10专属编码需求</x:v>
+      </x:c>
+      <x:c r="D224" s="83" t="str">
+        <x:v>件</x:v>
+      </x:c>
+      <x:c r="E224" s="83" t="n">
+        <x:v>464</x:v>
+      </x:c>
+      <x:c r="F224" s="83" t="n">
+        <x:v>464</x:v>
+      </x:c>
+      <x:c r="G224" s="83" t="n">
+        <x:v>464</x:v>
+      </x:c>
+      <x:c r="H224" s="115" t="str">
+        <x:v>已确认</x:v>
+      </x:c>
+      <x:c r="I224" s="94" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="J224" s="84" t="str">
+        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.1_编码阶段分配.xlsx＋装备素材套装代码表.xlsx＋材料编码数据库.xlsx</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="225" ht="36" customHeight="1">
+      <x:c r="A225" s="85" t="str">
+        <x:v>EL-PARAM-C3C10-CODE-ALLOCATED</x:v>
+      </x:c>
+      <x:c r="B225" s="86" t="str">
+        <x:v>编码资源</x:v>
+      </x:c>
+      <x:c r="C225" s="86" t="str">
+        <x:v>C3—C10已规划专属来源码</x:v>
+      </x:c>
+      <x:c r="D225" s="86" t="str">
+        <x:v>个</x:v>
+      </x:c>
+      <x:c r="E225" s="86" t="n">
+        <x:v>342</x:v>
+      </x:c>
+      <x:c r="F225" s="86" t="n">
+        <x:v>342</x:v>
+      </x:c>
+      <x:c r="G225" s="86" t="n">
+        <x:v>342</x:v>
+      </x:c>
+      <x:c r="H225" s="116" t="str">
+        <x:v>阶段分配完成</x:v>
+      </x:c>
+      <x:c r="I225" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="J225" s="87" t="str">
+        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.1_编码阶段分配.xlsx＋装备素材套装代码表.xlsx＋材料编码数据库.xlsx</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="226" ht="36" customHeight="1">
+      <x:c r="A226" s="85" t="str">
+        <x:v>EL-PARAM-C3C10-CODE-GAP</x:v>
+      </x:c>
+      <x:c r="B226" s="86" t="str">
+        <x:v>编码资源</x:v>
+      </x:c>
+      <x:c r="C226" s="86" t="str">
+        <x:v>C3—C10专属来源码缺口</x:v>
+      </x:c>
+      <x:c r="D226" s="86" t="str">
+        <x:v>个</x:v>
+      </x:c>
+      <x:c r="E226" s="86" t="n">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="F226" s="86" t="n">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="G226" s="86" t="n">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="H226" s="116" t="str">
+        <x:v>待用户补码</x:v>
+      </x:c>
+      <x:c r="I226" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="J226" s="87" t="str">
+        <x:v>武器60＋衣服51＋斗笠11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="227" ht="36" customHeight="1">
+      <x:c r="A227" s="85" t="str">
+        <x:v>EL-PARAM-C3C10-WEAPON-GAP</x:v>
+      </x:c>
+      <x:c r="B227" s="86" t="str">
+        <x:v>编码资源</x:v>
+      </x:c>
+      <x:c r="C227" s="86" t="str">
+        <x:v>武器来源码缺口</x:v>
+      </x:c>
+      <x:c r="D227" s="86" t="str">
+        <x:v>个</x:v>
+      </x:c>
+      <x:c r="E227" s="86" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F227" s="86" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="G227" s="86" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="H227" s="116" t="str">
+        <x:v>待用户补码</x:v>
+      </x:c>
+      <x:c r="I227" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="J227" s="87" t="str">
+        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.1_编码阶段分配.xlsx＋装备素材套装代码表.xlsx＋材料编码数据库.xlsx</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="228" ht="36" customHeight="1">
+      <x:c r="A228" s="85" t="str">
+        <x:v>EL-PARAM-C3C10-CLOTH-GAP</x:v>
+      </x:c>
+      <x:c r="B228" s="86" t="str">
+        <x:v>编码资源</x:v>
+      </x:c>
+      <x:c r="C228" s="86" t="str">
+        <x:v>衣服来源码缺口</x:v>
+      </x:c>
+      <x:c r="D228" s="86" t="str">
+        <x:v>个</x:v>
+      </x:c>
+      <x:c r="E228" s="86" t="n">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="F228" s="86" t="n">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="G228" s="86" t="n">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="H228" s="116" t="str">
+        <x:v>待用户补码</x:v>
+      </x:c>
+      <x:c r="I228" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="J228" s="87" t="str">
+        <x:v>严格按男衣服StdMode10；女衣服未合池</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="229" ht="36" customHeight="1">
+      <x:c r="A229" s="85" t="str">
+        <x:v>EL-PARAM-C3C10-HAT-GAP</x:v>
+      </x:c>
+      <x:c r="B229" s="86" t="str">
+        <x:v>编码资源</x:v>
+      </x:c>
+      <x:c r="C229" s="86" t="str">
+        <x:v>斗笠来源码缺口</x:v>
+      </x:c>
+      <x:c r="D229" s="86" t="str">
+        <x:v>个</x:v>
+      </x:c>
+      <x:c r="E229" s="86" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="F229" s="86" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="G229" s="86" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H229" s="116" t="str">
+        <x:v>待用户补码</x:v>
+      </x:c>
+      <x:c r="I229" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="J229" s="87" t="str">
+        <x:v>面巾StdMode16／位置13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="230" ht="36" customHeight="1">
+      <x:c r="A230" s="85" t="str">
+        <x:v>EL-PARAM-C3C10-COLLECT-IDX</x:v>
+      </x:c>
+      <x:c r="B230" s="86" t="str">
+        <x:v>编码资源</x:v>
+      </x:c>
+      <x:c r="C230" s="86" t="str">
+        <x:v>大陆收藏材料已规划Idx</x:v>
+      </x:c>
+      <x:c r="D230" s="86" t="str">
+        <x:v>个</x:v>
+      </x:c>
+      <x:c r="E230" s="86" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F230" s="86" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G230" s="86" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H230" s="116" t="str">
+        <x:v>规划锁定／未入库</x:v>
+      </x:c>
+      <x:c r="I230" s="95" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="J230" s="87" t="str">
+        <x:v>972—979</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="231" ht="36" customHeight="1">
+      <x:c r="A231" s="88" t="str">
+        <x:v>EL-PARAM-C3C10-COLLECT-LOOKS-GAP</x:v>
+      </x:c>
+      <x:c r="B231" s="89" t="str">
+        <x:v>编码资源</x:v>
+      </x:c>
+      <x:c r="C231" s="89" t="str">
+        <x:v>大陆收藏材料Items Looks缺口</x:v>
+      </x:c>
+      <x:c r="D231" s="89" t="str">
+        <x:v>个</x:v>
+      </x:c>
+      <x:c r="E231" s="89" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F231" s="89" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G231" s="89" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H231" s="117" t="str">
+        <x:v>待用户/平台提供</x:v>
+      </x:c>
+      <x:c r="I231" s="96" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="J231" s="90" t="str">
+        <x:v>不得使用与装备资源重叠的6463—6470</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -14407,16 +14792,42 @@
         <x:v>第3—10大陆</x:v>
       </x:c>
       <x:c r="E25" s="112" t="str">
-        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.0.xlsx</x:v>
+        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.1_编码阶段分配.xlsx</x:v>
       </x:c>
       <x:c r="F25" s="114" t="n">
         <x:v>46267</x:v>
       </x:c>
       <x:c r="G25" s="112" t="str">
-        <x:v>464怪逐一对应；来源编号与正式属性待后续施工</x:v>
+        <x:v>464怪逐一对应；342件已规划来源编号，122件待补同部位码；正式属性待后续施工</x:v>
       </x:c>
       <x:c r="H25" s="113" t="str">
-        <x:v>结构定稿／待分配编码</x:v>
+        <x:v>结构定稿／编码阶段分配</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="46" customHeight="1">
+      <x:c r="A26" s="111" t="str">
+        <x:v>EL-EQUIP-C3C10-CODE-001</x:v>
+      </x:c>
+      <x:c r="B26" s="112" t="str">
+        <x:v>定向专属编码</x:v>
+      </x:c>
+      <x:c r="C26" s="112" t="str">
+        <x:v>第3—10大陆464件一怪一专属</x:v>
+      </x:c>
+      <x:c r="D26" s="112" t="str">
+        <x:v>第3—10大陆</x:v>
+      </x:c>
+      <x:c r="E26" s="112" t="str">
+        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.1_编码阶段分配.xlsx＋装备素材套装代码表.xlsx＋材料编码数据库.xlsx</x:v>
+      </x:c>
+      <x:c r="F26" s="114" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="G26" s="112" t="str">
+        <x:v>342件已锁定来源编号；122件缺码详见09_编码缺口</x:v>
+      </x:c>
+      <x:c r="H26" s="113" t="str">
+        <x:v>阶段分配／未入库</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -15635,7 +16046,7 @@
         <x:v>46256</x:v>
       </x:c>
       <x:c r="G14" s="62" t="str">
-        <x:v>972—983预留；793/794/802不变；只写Items图库；6398—6462不得作为新装备Items来源编号</x:v>
+        <x:v>Idx 972—979已转为批次B规划，Items Looks待补；980—983继续冻结；793/794/802不变；只写Items图库；6398—6462不得作为新装备Items来源编号</x:v>
       </x:c>
       <x:c r="H14" s="63" t="str">
         <x:v>原件已接续／65条逐行通过／游戏内待验收</x:v>
@@ -15681,16 +16092,42 @@
         <x:v>按大陆来源</x:v>
       </x:c>
       <x:c r="E16" s="89" t="str">
-        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.0.xlsx</x:v>
+        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.1_编码阶段分配.xlsx</x:v>
       </x:c>
       <x:c r="F16" s="96" t="n">
         <x:v>46267</x:v>
       </x:c>
       <x:c r="G16" s="89" t="str">
-        <x:v>既有材料Idx 916—971；收藏材料代码待取</x:v>
+        <x:v>既有材料Idx 916—971；收藏材料Idx 972—979已规划，Items Looks待补</x:v>
       </x:c>
       <x:c r="H16" s="90" t="str">
-        <x:v>名称与来源定稿／概率待算</x:v>
+        <x:v>名称与来源定稿／Idx已规划／概率待算</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="46" customHeight="1">
+      <x:c r="A17" s="111" t="str">
+        <x:v>EL-DROP-C3C10-COLLECT-CODE-001</x:v>
+      </x:c>
+      <x:c r="B17" s="112" t="str">
+        <x:v>第3—10大陆全部怪物</x:v>
+      </x:c>
+      <x:c r="C17" s="112" t="str">
+        <x:v>8件大陆收藏材料</x:v>
+      </x:c>
+      <x:c r="D17" s="112" t="str">
+        <x:v>Idx 972—979已规划；Looks待补</x:v>
+      </x:c>
+      <x:c r="E17" s="112" t="str">
+        <x:v>第3至10大陆_怪物专属与材料来源总账_V1.1_编码阶段分配.xlsx＋装备素材套装代码表.xlsx＋材料编码数据库.xlsx</x:v>
+      </x:c>
+      <x:c r="F17" s="114" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="G17" s="112" t="str">
+        <x:v>只记录编码规划，不代表掉落概率或平台部署</x:v>
+      </x:c>
+      <x:c r="H17" s="113" t="str">
+        <x:v>编码阶段／概率待算</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>